<commit_message>
v.0.27 Add Admin Panel Update AdminDashboardController
</commit_message>
<xml_diff>
--- a/docs/PSP_OnlineShop.xlsx
+++ b/docs/PSP_OnlineShop.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="2"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="PSP" sheetId="1" state="visible" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="246">
   <si>
     <t>Projektstrukturplan</t>
   </si>
@@ -341,7 +341,7 @@
     <t>Status:</t>
   </si>
   <si>
-    <t>offen</t>
+    <t>fertig</t>
   </si>
   <si>
     <t xml:space="preserve">Abgeschlossen am:</t>
@@ -464,6 +464,9 @@
   </si>
   <si>
     <t xml:space="preserve">– H2-Kompatibilität mit Flyway-Migrationen prüfen (MySQL-spezifische SQL-Syntax ggf. anpassen)</t>
+  </si>
+  <si>
+    <t>offen</t>
   </si>
   <si>
     <t xml:space="preserve">End-to-End-Integrationstests für kritische Flows (Checkout, Auth), Testszenarien /T01/–/T12/ aus dem Lastenheft manuell durchführen, Testprotokolle in PSP.xlsx ausfüllen.</t>
@@ -796,10 +799,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd\.mm\.yyyy"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="7">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -814,12 +818,10 @@
     <font>
       <b/>
       <sz val="10.000000"/>
-      <color indexed="64"/>
       <name val="Arial"/>
     </font>
     <font>
       <sz val="10.000000"/>
-      <color indexed="64"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -838,15 +840,6 @@
       <b/>
       <sz val="13.000000"/>
       <color indexed="65"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10.000000"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10.000000"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -952,7 +945,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="54">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1032,6 +1025,12 @@
     <xf fontId="3" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf fontId="3" fillId="8" borderId="1" numFmtId="165" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="8" borderId="1" numFmtId="164" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf fontId="3" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1053,6 +1052,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="3" fillId="3" borderId="1" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="8" borderId="1" numFmtId="164" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="3" fillId="10" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1088,10 +1090,10 @@
     <xf fontId="6" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="7" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="8" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2143,7 +2145,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="16"/>
     <col customWidth="1" min="2" max="2" width="60"/>
@@ -2219,7 +2221,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="12" ht="39.75" customHeight="1">
+    <row r="12" ht="33.5" customHeight="1">
       <c r="A12" s="27" t="s">
         <v>98</v>
       </c>
@@ -2239,7 +2241,9 @@
       <c r="A14" s="27" t="s">
         <v>102</v>
       </c>
-      <c r="B14" s="29"/>
+      <c r="B14" s="29">
+        <v>46170</v>
+      </c>
     </row>
     <row r="15" ht="19.5" customHeight="1">
       <c r="A15" s="27" t="s">
@@ -2253,17 +2257,19 @@
       <c r="A16" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="B16" s="29"/>
+      <c r="B16" s="30">
+        <v>46171</v>
+      </c>
     </row>
     <row r="17" ht="19.5" customHeight="1">
       <c r="A17" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="B17" s="29"/>
+      <c r="B17" s="31"/>
     </row>
     <row r="18" ht="7.5" customHeight="1">
-      <c r="A18" s="30"/>
-      <c r="B18" s="30"/>
+      <c r="A18" s="32"/>
+      <c r="B18" s="32"/>
     </row>
     <row r="19" ht="37.799999999999997" customHeight="1">
       <c r="A19" s="27" t="s">
@@ -2325,7 +2331,9 @@
       <c r="A26" s="27" t="s">
         <v>102</v>
       </c>
-      <c r="B26" s="29"/>
+      <c r="B26" s="29">
+        <v>46174</v>
+      </c>
     </row>
     <row r="27" ht="19.5" customHeight="1">
       <c r="A27" s="27" t="s">
@@ -2339,17 +2347,19 @@
       <c r="A28" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="B28" s="29"/>
+      <c r="B28" s="29">
+        <v>46177</v>
+      </c>
     </row>
     <row r="29" ht="19.5" customHeight="1">
       <c r="A29" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="B29" s="29"/>
+      <c r="B29" s="31"/>
     </row>
     <row r="30" ht="7.5" customHeight="1">
-      <c r="A30" s="30"/>
-      <c r="B30" s="30"/>
+      <c r="A30" s="32"/>
+      <c r="B30" s="32"/>
     </row>
     <row r="31" ht="19.5" customHeight="1">
       <c r="A31" s="27" t="s">
@@ -2411,7 +2421,9 @@
       <c r="A38" s="27" t="s">
         <v>102</v>
       </c>
-      <c r="B38" s="29"/>
+      <c r="B38" s="29">
+        <v>46178</v>
+      </c>
     </row>
     <row r="39" ht="19.5" customHeight="1">
       <c r="A39" s="27" t="s">
@@ -2425,17 +2437,19 @@
       <c r="A40" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="B40" s="29"/>
+      <c r="B40" s="30">
+        <v>46180</v>
+      </c>
     </row>
     <row r="41" ht="19.5" customHeight="1">
       <c r="A41" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="B41" s="29"/>
+      <c r="B41" s="31"/>
     </row>
     <row r="42" ht="7.5" customHeight="1">
-      <c r="A42" s="30"/>
-      <c r="B42" s="30"/>
+      <c r="A42" s="32"/>
+      <c r="B42" s="32"/>
     </row>
     <row r="43" ht="36" customHeight="1">
       <c r="A43" s="27" t="s">
@@ -2497,7 +2511,9 @@
       <c r="A50" s="27" t="s">
         <v>102</v>
       </c>
-      <c r="B50" s="29"/>
+      <c r="B50" s="29">
+        <v>46180</v>
+      </c>
     </row>
     <row r="51" ht="19.5" customHeight="1">
       <c r="A51" s="27" t="s">
@@ -2511,17 +2527,19 @@
       <c r="A52" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="B52" s="29"/>
+      <c r="B52" s="29">
+        <v>46181</v>
+      </c>
     </row>
     <row r="53" ht="19.5" customHeight="1">
       <c r="A53" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="B53" s="29"/>
+      <c r="B53" s="31"/>
     </row>
     <row r="54" ht="7.5" customHeight="1">
-      <c r="A54" s="30"/>
-      <c r="B54" s="30"/>
+      <c r="A54" s="32"/>
+      <c r="B54" s="32"/>
     </row>
     <row r="55" ht="19.5" customHeight="1">
       <c r="A55" s="27" t="s">
@@ -2583,7 +2601,9 @@
       <c r="A62" s="27" t="s">
         <v>102</v>
       </c>
-      <c r="B62" s="29"/>
+      <c r="B62" s="29">
+        <v>46181</v>
+      </c>
     </row>
     <row r="63" ht="19.5" customHeight="1">
       <c r="A63" s="27" t="s">
@@ -2597,17 +2617,19 @@
       <c r="A64" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="B64" s="29"/>
+      <c r="B64" s="30">
+        <v>46182</v>
+      </c>
     </row>
     <row r="65" ht="19.5" customHeight="1">
       <c r="A65" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="B65" s="29"/>
+      <c r="B65" s="31"/>
     </row>
     <row r="66" ht="7.5" customHeight="1">
-      <c r="A66" s="30"/>
-      <c r="B66" s="30"/>
+      <c r="A66" s="32"/>
+      <c r="B66" s="32"/>
     </row>
     <row r="67" ht="19.5" customHeight="1">
       <c r="A67" s="27" t="s">
@@ -2669,7 +2691,9 @@
       <c r="A74" s="27" t="s">
         <v>102</v>
       </c>
-      <c r="B74" s="29"/>
+      <c r="B74" s="30">
+        <v>46182</v>
+      </c>
     </row>
     <row r="75" ht="19.5" customHeight="1">
       <c r="A75" s="27" t="s">
@@ -2683,17 +2707,19 @@
       <c r="A76" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="B76" s="29"/>
+      <c r="B76" s="30">
+        <v>46183</v>
+      </c>
     </row>
     <row r="77" ht="19.5" customHeight="1">
       <c r="A77" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="B77" s="29"/>
+      <c r="B77" s="31"/>
     </row>
     <row r="78" ht="7.5" customHeight="1">
-      <c r="A78" s="30"/>
-      <c r="B78" s="30"/>
+      <c r="A78" s="32"/>
+      <c r="B78" s="32"/>
     </row>
     <row r="79" ht="31.199999999999999" customHeight="1">
       <c r="A79" s="27" t="s">
@@ -2755,7 +2781,9 @@
       <c r="A86" s="27" t="s">
         <v>102</v>
       </c>
-      <c r="B86" s="29"/>
+      <c r="B86" s="30">
+        <v>46183</v>
+      </c>
     </row>
     <row r="87" ht="19.5" customHeight="1">
       <c r="A87" s="27" t="s">
@@ -2769,17 +2797,19 @@
       <c r="A88" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="B88" s="29"/>
+      <c r="B88" s="30">
+        <v>46184</v>
+      </c>
     </row>
     <row r="89" ht="19.5" customHeight="1">
       <c r="A89" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="B89" s="29"/>
+      <c r="B89" s="31"/>
     </row>
     <row r="90" ht="7.5" customHeight="1">
-      <c r="A90" s="30"/>
-      <c r="B90" s="30"/>
+      <c r="A90" s="32"/>
+      <c r="B90" s="32"/>
     </row>
     <row r="91" ht="19.5" customHeight="1">
       <c r="A91" s="27" t="s">
@@ -2841,31 +2871,33 @@
       <c r="A98" s="27" t="s">
         <v>102</v>
       </c>
-      <c r="B98" s="29"/>
+      <c r="B98" s="30">
+        <v>46176</v>
+      </c>
     </row>
     <row r="99" ht="19.5" customHeight="1">
       <c r="A99" s="27" t="s">
         <v>103</v>
       </c>
       <c r="B99" s="28" t="s">
-        <v>104</v>
+        <v>137</v>
       </c>
     </row>
     <row r="100" ht="19.5" customHeight="1">
       <c r="A100" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="B100" s="29"/>
+      <c r="B100" s="31"/>
     </row>
     <row r="101" ht="19.5" customHeight="1">
       <c r="A101" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="B101" s="29"/>
+      <c r="B101" s="31"/>
     </row>
     <row r="102" ht="16.800000000000001" customHeight="1">
-      <c r="A102" s="30"/>
-      <c r="B102" s="30"/>
+      <c r="A102" s="32"/>
+      <c r="B102" s="32"/>
     </row>
     <row r="103" ht="19.5" customHeight="1">
       <c r="A103" s="27" t="s">
@@ -2888,7 +2920,7 @@
         <v>92</v>
       </c>
       <c r="B105" s="28" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="106" ht="39.75" customHeight="1">
@@ -2896,7 +2928,7 @@
         <v>94</v>
       </c>
       <c r="B106" s="28" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="107" ht="19.5" customHeight="1">
@@ -2904,7 +2936,7 @@
         <v>96</v>
       </c>
       <c r="B107" s="28" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="108" ht="39.75" customHeight="1">
@@ -2912,7 +2944,7 @@
         <v>98</v>
       </c>
       <c r="B108" s="28" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="109" ht="19.5" customHeight="1">
@@ -2927,44 +2959,46 @@
       <c r="A110" s="27" t="s">
         <v>102</v>
       </c>
-      <c r="B110" s="29"/>
+      <c r="B110" s="29">
+        <v>46182</v>
+      </c>
     </row>
     <row r="111" ht="19.5" customHeight="1">
       <c r="A111" s="27" t="s">
         <v>103</v>
       </c>
       <c r="B111" s="28" t="s">
-        <v>104</v>
+        <v>137</v>
       </c>
     </row>
     <row r="112" ht="19.5" customHeight="1">
       <c r="A112" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="B112" s="29"/>
+      <c r="B112" s="31"/>
     </row>
     <row r="113" ht="19.5" customHeight="1">
       <c r="A113" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="B113" s="29"/>
+      <c r="B113" s="31"/>
     </row>
     <row r="114" ht="7.5" customHeight="1">
-      <c r="A114" s="30"/>
-      <c r="B114" s="30"/>
+      <c r="A114" s="32"/>
+      <c r="B114" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="A54:B54"/>
     <mergeCell ref="A66:B66"/>
     <mergeCell ref="A78:B78"/>
     <mergeCell ref="A90:B90"/>
     <mergeCell ref="A102:B102"/>
     <mergeCell ref="A114:B114"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="A54:B54"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51181102362204689" footer="0.51181102362204689"/>
@@ -2975,7 +3009,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="7"/>
     <col customWidth="1" min="2" max="2" width="10"/>
@@ -2989,7 +3023,7 @@
   <sheetData>
     <row r="1" ht="17.25" customHeight="1">
       <c r="A1" s="24" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B1" s="24"/>
       <c r="C1" s="24"/>
@@ -3011,7 +3045,7 @@
       <c r="D3" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="31">
+      <c r="E3" s="33">
         <v>46168</v>
       </c>
     </row>
@@ -3025,7 +3059,7 @@
       <c r="D4" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="31">
+      <c r="E4" s="33">
         <v>46220</v>
       </c>
     </row>
@@ -3047,7 +3081,7 @@
       <c r="A6" s="25"/>
       <c r="B6" s="26"/>
       <c r="D6" s="25" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E6" s="26">
         <v>40</v>
@@ -3057,7 +3091,7 @@
       <c r="A7" s="25"/>
       <c r="B7" s="26"/>
       <c r="D7" s="25" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E7" s="26">
         <v>40</v>
@@ -3067,7 +3101,7 @@
       <c r="A8" s="25"/>
       <c r="B8" s="26"/>
       <c r="D8" s="25" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E8" s="26">
         <f>E7-E6</f>
@@ -3082,28 +3116,28 @@
         <v>12</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="10" ht="19.5" customHeight="1">
@@ -3119,20 +3153,20 @@
       <c r="D10" s="18">
         <v>3</v>
       </c>
-      <c r="E10" s="32">
+      <c r="E10" s="34">
         <v>46168</v>
       </c>
-      <c r="F10" s="32">
+      <c r="F10" s="34">
         <v>46170</v>
       </c>
-      <c r="G10" s="33">
+      <c r="G10" s="35">
         <v>46169</v>
       </c>
-      <c r="H10" s="34">
+      <c r="H10" s="36">
         <f t="shared" ref="H10:H32" si="0">IF(ISBLANK(G10),"",G10-F10)</f>
         <v>-1</v>
       </c>
-      <c r="I10" s="35" t="str">
+      <c r="I10" s="37" t="str">
         <f t="shared" ref="I10:I32" si="1">IF(ISBLANK(G10),"offen","fertig")</f>
         <v>fertig</v>
       </c>
@@ -3146,25 +3180,25 @@
         <v>20</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D11" s="18">
         <v>3</v>
       </c>
-      <c r="E11" s="32">
+      <c r="E11" s="34">
         <v>46168</v>
       </c>
-      <c r="F11" s="32">
+      <c r="F11" s="34">
         <v>46170</v>
       </c>
-      <c r="G11" s="33">
+      <c r="G11" s="35">
         <v>46170</v>
       </c>
-      <c r="H11" s="34">
+      <c r="H11" s="36">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I11" s="35" t="str">
+      <c r="I11" s="37" t="str">
         <f t="shared" si="1"/>
         <v>fertig</v>
       </c>
@@ -3178,30 +3212,30 @@
         <v>23</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D12" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="E12" s="36">
+      <c r="E12" s="38">
         <v>46171</v>
       </c>
-      <c r="F12" s="36">
+      <c r="F12" s="38">
         <v>46171</v>
       </c>
-      <c r="G12" s="33">
+      <c r="G12" s="35">
         <v>46171</v>
       </c>
-      <c r="H12" s="34">
+      <c r="H12" s="36">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I12" s="35" t="str">
+      <c r="I12" s="37" t="str">
         <f t="shared" si="1"/>
         <v>fertig</v>
       </c>
       <c r="J12" s="14" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="13" ht="19.5" customHeight="1">
@@ -3217,20 +3251,20 @@
       <c r="D13" s="18">
         <v>2</v>
       </c>
-      <c r="E13" s="32">
+      <c r="E13" s="34">
         <v>46171</v>
       </c>
-      <c r="F13" s="32">
+      <c r="F13" s="34">
         <v>46174</v>
       </c>
-      <c r="G13" s="33">
+      <c r="G13" s="35">
         <v>46171</v>
       </c>
-      <c r="H13" s="34">
+      <c r="H13" s="36">
         <f t="shared" si="0"/>
         <v>-3</v>
       </c>
-      <c r="I13" s="35" t="str">
+      <c r="I13" s="37" t="str">
         <f t="shared" si="1"/>
         <v>fertig</v>
       </c>
@@ -3249,25 +3283,25 @@
       <c r="D14" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="E14" s="36">
+      <c r="E14" s="38">
         <v>46175</v>
       </c>
-      <c r="F14" s="36">
+      <c r="F14" s="38">
         <v>46175</v>
       </c>
-      <c r="G14" s="33">
+      <c r="G14" s="35">
         <v>46171</v>
       </c>
-      <c r="H14" s="34">
+      <c r="H14" s="36">
         <f t="shared" si="0"/>
         <v>-4</v>
       </c>
-      <c r="I14" s="35" t="str">
+      <c r="I14" s="37" t="str">
         <f t="shared" si="1"/>
         <v>fertig</v>
       </c>
       <c r="J14" s="14" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="15" ht="19.5" customHeight="1">
@@ -3278,25 +3312,25 @@
         <v>33</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D15" s="18">
         <v>3</v>
       </c>
-      <c r="E15" s="32">
+      <c r="E15" s="34">
         <v>46175</v>
       </c>
-      <c r="F15" s="32">
+      <c r="F15" s="34">
         <v>46178</v>
       </c>
-      <c r="G15" s="33">
+      <c r="G15" s="35">
         <v>46172</v>
       </c>
-      <c r="H15" s="34">
+      <c r="H15" s="36">
         <f t="shared" si="0"/>
         <v>-6</v>
       </c>
-      <c r="I15" s="35" t="str">
+      <c r="I15" s="37" t="str">
         <f t="shared" si="1"/>
         <v>fertig</v>
       </c>
@@ -3315,25 +3349,25 @@
       <c r="D16" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="E16" s="32">
+      <c r="E16" s="34">
         <v>46178</v>
       </c>
-      <c r="F16" s="32">
+      <c r="F16" s="34">
         <v>46178</v>
       </c>
-      <c r="G16" s="33">
+      <c r="G16" s="35">
         <v>46174</v>
       </c>
-      <c r="H16" s="34">
+      <c r="H16" s="36">
         <f t="shared" si="0"/>
         <v>-4</v>
       </c>
-      <c r="I16" s="35" t="str">
+      <c r="I16" s="37" t="str">
         <f t="shared" si="1"/>
         <v>fertig</v>
       </c>
       <c r="J16" s="19" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="17" ht="19.5" customHeight="1">
@@ -3349,20 +3383,20 @@
       <c r="D17" s="8">
         <v>3</v>
       </c>
-      <c r="E17" s="37">
+      <c r="E17" s="39">
         <v>46178</v>
       </c>
-      <c r="F17" s="37">
+      <c r="F17" s="39">
         <v>46182</v>
       </c>
-      <c r="G17" s="33">
+      <c r="G17" s="35">
         <v>46171</v>
       </c>
-      <c r="H17" s="34">
+      <c r="H17" s="36">
         <f t="shared" si="0"/>
         <v>-11</v>
       </c>
-      <c r="I17" s="35" t="str">
+      <c r="I17" s="37" t="str">
         <f t="shared" si="1"/>
         <v>fertig</v>
       </c>
@@ -3381,20 +3415,20 @@
       <c r="D18" s="8">
         <v>4</v>
       </c>
-      <c r="E18" s="37">
+      <c r="E18" s="39">
         <v>46182</v>
       </c>
-      <c r="F18" s="37">
+      <c r="F18" s="39">
         <v>46185</v>
       </c>
-      <c r="G18" s="33">
-        <v>46146</v>
-      </c>
-      <c r="H18" s="34">
+      <c r="G18" s="35">
+        <v>46177</v>
+      </c>
+      <c r="H18" s="36">
         <f t="shared" si="0"/>
-        <v>-39</v>
-      </c>
-      <c r="I18" s="35" t="str">
+        <v>-8</v>
+      </c>
+      <c r="I18" s="37" t="str">
         <f t="shared" si="1"/>
         <v>fertig</v>
       </c>
@@ -3413,20 +3447,22 @@
       <c r="D19" s="8">
         <v>4</v>
       </c>
-      <c r="E19" s="37">
+      <c r="E19" s="39">
         <v>46185</v>
       </c>
-      <c r="F19" s="37">
+      <c r="F19" s="39">
         <v>46190</v>
       </c>
-      <c r="G19" s="33"/>
-      <c r="H19" s="34" t="str">
+      <c r="G19" s="35">
+        <v>46180</v>
+      </c>
+      <c r="H19" s="36">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I19" s="35" t="str">
+        <v>-10</v>
+      </c>
+      <c r="I19" s="37" t="str">
         <f t="shared" si="1"/>
-        <v>offen</v>
+        <v>fertig</v>
       </c>
       <c r="J19" s="9"/>
     </row>
@@ -3443,20 +3479,22 @@
       <c r="D20" s="8">
         <v>3</v>
       </c>
-      <c r="E20" s="37">
+      <c r="E20" s="39">
         <v>46190</v>
       </c>
-      <c r="F20" s="37">
+      <c r="F20" s="39">
         <v>46192</v>
       </c>
-      <c r="G20" s="33"/>
-      <c r="H20" s="34" t="str">
+      <c r="G20" s="40">
+        <v>46181</v>
+      </c>
+      <c r="H20" s="36">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I20" s="35" t="str">
+        <v>-11</v>
+      </c>
+      <c r="I20" s="37" t="str">
         <f t="shared" si="1"/>
-        <v>offen</v>
+        <v>fertig</v>
       </c>
       <c r="J20" s="9"/>
     </row>
@@ -3473,23 +3511,25 @@
       <c r="D21" s="8">
         <v>4</v>
       </c>
-      <c r="E21" s="37">
+      <c r="E21" s="39">
         <v>46192</v>
       </c>
-      <c r="F21" s="37">
+      <c r="F21" s="39">
         <v>46198</v>
       </c>
-      <c r="G21" s="33"/>
-      <c r="H21" s="34" t="str">
+      <c r="G21" s="35">
+        <v>46182</v>
+      </c>
+      <c r="H21" s="36">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I21" s="35" t="str">
+        <v>-16</v>
+      </c>
+      <c r="I21" s="37" t="str">
         <f t="shared" si="1"/>
-        <v>offen</v>
+        <v>fertig</v>
       </c>
       <c r="J21" s="9" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="22" ht="19.5" customHeight="1">
@@ -3505,20 +3545,22 @@
       <c r="D22" s="8">
         <v>4</v>
       </c>
-      <c r="E22" s="37">
+      <c r="E22" s="39">
         <v>46198</v>
       </c>
-      <c r="F22" s="37">
+      <c r="F22" s="39">
         <v>46204</v>
       </c>
-      <c r="G22" s="33"/>
-      <c r="H22" s="34" t="str">
+      <c r="G22" s="35">
+        <v>46183</v>
+      </c>
+      <c r="H22" s="36">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I22" s="35" t="str">
+        <v>-21</v>
+      </c>
+      <c r="I22" s="37" t="str">
         <f t="shared" si="1"/>
-        <v>offen</v>
+        <v>fertig</v>
       </c>
       <c r="J22" s="9"/>
     </row>
@@ -3535,20 +3577,22 @@
       <c r="D23" s="8">
         <v>2</v>
       </c>
-      <c r="E23" s="37">
+      <c r="E23" s="39">
         <v>46204</v>
       </c>
-      <c r="F23" s="37">
+      <c r="F23" s="39">
         <v>46206</v>
       </c>
-      <c r="G23" s="33"/>
-      <c r="H23" s="34" t="str">
+      <c r="G23" s="35">
+        <v>46184</v>
+      </c>
+      <c r="H23" s="36">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I23" s="35" t="str">
+        <v>-22</v>
+      </c>
+      <c r="I23" s="37" t="str">
         <f t="shared" si="1"/>
-        <v>offen</v>
+        <v>fertig</v>
       </c>
       <c r="J23" s="9"/>
     </row>
@@ -3560,28 +3604,28 @@
         <v>60</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D24" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="E24" s="36">
+      <c r="E24" s="38">
         <v>46206</v>
       </c>
-      <c r="F24" s="36">
+      <c r="F24" s="38">
         <v>46206</v>
       </c>
-      <c r="G24" s="33"/>
-      <c r="H24" s="34" t="str">
+      <c r="G24" s="35"/>
+      <c r="H24" s="36" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I24" s="35" t="str">
+      <c r="I24" s="37" t="str">
         <f t="shared" si="1"/>
         <v>offen</v>
       </c>
       <c r="J24" s="14" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
     </row>
     <row r="25" ht="19.5" customHeight="1">
@@ -3597,18 +3641,18 @@
       <c r="D25" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="E25" s="32">
+      <c r="E25" s="34">
         <v>46206</v>
       </c>
-      <c r="F25" s="32">
+      <c r="F25" s="34">
         <v>46206</v>
       </c>
-      <c r="G25" s="33"/>
-      <c r="H25" s="34" t="str">
+      <c r="G25" s="35"/>
+      <c r="H25" s="36" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I25" s="35" t="str">
+      <c r="I25" s="37" t="str">
         <f t="shared" si="1"/>
         <v>offen</v>
       </c>
@@ -3622,23 +3666,23 @@
         <v>66</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D26" s="8">
         <v>2</v>
       </c>
-      <c r="E26" s="37">
+      <c r="E26" s="39">
         <v>46206</v>
       </c>
-      <c r="F26" s="37">
+      <c r="F26" s="39">
         <v>46210</v>
       </c>
-      <c r="G26" s="33"/>
-      <c r="H26" s="34" t="str">
+      <c r="G26" s="35"/>
+      <c r="H26" s="36" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I26" s="35" t="str">
+      <c r="I26" s="37" t="str">
         <f t="shared" si="1"/>
         <v>offen</v>
       </c>
@@ -3657,18 +3701,18 @@
       <c r="D27" s="8">
         <v>2</v>
       </c>
-      <c r="E27" s="37">
+      <c r="E27" s="39">
         <v>46210</v>
       </c>
-      <c r="F27" s="37">
+      <c r="F27" s="39">
         <v>46212</v>
       </c>
-      <c r="G27" s="33"/>
-      <c r="H27" s="34" t="str">
+      <c r="G27" s="35"/>
+      <c r="H27" s="36" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I27" s="35" t="str">
+      <c r="I27" s="37" t="str">
         <f t="shared" si="1"/>
         <v>offen</v>
       </c>
@@ -3687,18 +3731,18 @@
       <c r="D28" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="E28" s="36">
+      <c r="E28" s="38">
         <v>46212</v>
       </c>
-      <c r="F28" s="36">
+      <c r="F28" s="38">
         <v>46212</v>
       </c>
-      <c r="G28" s="33"/>
-      <c r="H28" s="34" t="str">
+      <c r="G28" s="35"/>
+      <c r="H28" s="36" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I28" s="35" t="str">
+      <c r="I28" s="37" t="str">
         <f t="shared" si="1"/>
         <v>offen</v>
       </c>
@@ -3712,23 +3756,23 @@
         <v>75</v>
       </c>
       <c r="C29" s="17" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D29" s="18">
         <v>1</v>
       </c>
-      <c r="E29" s="32">
+      <c r="E29" s="34">
         <v>46212</v>
       </c>
-      <c r="F29" s="32">
+      <c r="F29" s="34">
         <v>46213</v>
       </c>
-      <c r="G29" s="33"/>
-      <c r="H29" s="34" t="str">
+      <c r="G29" s="35"/>
+      <c r="H29" s="36" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I29" s="35" t="str">
+      <c r="I29" s="37" t="str">
         <f t="shared" si="1"/>
         <v>offen</v>
       </c>
@@ -3747,18 +3791,18 @@
       <c r="D30" s="18">
         <v>1</v>
       </c>
-      <c r="E30" s="32">
+      <c r="E30" s="34">
         <v>46213</v>
       </c>
-      <c r="F30" s="32">
+      <c r="F30" s="34">
         <v>46216</v>
       </c>
-      <c r="G30" s="33"/>
-      <c r="H30" s="34" t="str">
+      <c r="G30" s="35"/>
+      <c r="H30" s="36" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I30" s="35" t="str">
+      <c r="I30" s="37" t="str">
         <f t="shared" si="1"/>
         <v>offen</v>
       </c>
@@ -3777,23 +3821,23 @@
       <c r="D31" s="13">
         <v>1</v>
       </c>
-      <c r="E31" s="36">
+      <c r="E31" s="38">
         <v>46216</v>
       </c>
-      <c r="F31" s="36">
+      <c r="F31" s="38">
         <v>46217</v>
       </c>
-      <c r="G31" s="33"/>
-      <c r="H31" s="34" t="str">
+      <c r="G31" s="35"/>
+      <c r="H31" s="36" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I31" s="35" t="str">
+      <c r="I31" s="37" t="str">
         <f t="shared" si="1"/>
         <v>offen</v>
       </c>
       <c r="J31" s="14" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="32" ht="19.5" customHeight="1">
@@ -3804,23 +3848,23 @@
         <v>85</v>
       </c>
       <c r="C32" s="12" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D32" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="E32" s="36">
+      <c r="E32" s="38">
         <v>46220</v>
       </c>
-      <c r="F32" s="36">
+      <c r="F32" s="38">
         <v>46220</v>
       </c>
-      <c r="G32" s="33"/>
-      <c r="H32" s="34" t="str">
+      <c r="G32" s="35"/>
+      <c r="H32" s="36" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I32" s="35" t="str">
+      <c r="I32" s="37" t="str">
         <f t="shared" si="1"/>
         <v>offen</v>
       </c>
@@ -3869,7 +3913,7 @@
   <sheetData>
     <row r="1" ht="17.25" customHeight="1">
       <c r="A1" s="24" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B1" s="24"/>
       <c r="C1" s="24"/>
@@ -3905,1007 +3949,1007 @@
         <v>11</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="8" ht="19.5" customHeight="1">
-      <c r="A8" s="38" t="s">
-        <v>169</v>
-      </c>
-      <c r="B8" s="39" t="s">
+      <c r="A8" s="41" t="s">
         <v>170</v>
       </c>
-      <c r="C8" s="33">
+      <c r="B8" s="42" t="s">
+        <v>171</v>
+      </c>
+      <c r="C8" s="35">
         <v>46176</v>
       </c>
-      <c r="D8" s="35" t="str">
-        <f>IF(ISBLANK(C8),"offen","fertig")</f>
+      <c r="D8" s="37" t="str">
+        <f t="shared" ref="D8:D9" si="2">IF(ISBLANK(C8),"offen","fertig")</f>
         <v>fertig</v>
       </c>
-      <c r="E8" s="40"/>
+      <c r="E8" s="43"/>
     </row>
     <row r="9" ht="19.5" customHeight="1">
       <c r="A9" s="8" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>172</v>
-      </c>
-      <c r="C9" s="33">
+        <v>173</v>
+      </c>
+      <c r="C9" s="35">
         <v>46177</v>
       </c>
-      <c r="D9" s="35" t="str">
-        <f>IF(ISBLANK(C9),"offen","fertig")</f>
+      <c r="D9" s="37" t="str">
+        <f t="shared" si="2"/>
         <v>fertig</v>
       </c>
-      <c r="E9" s="40"/>
+      <c r="E9" s="43"/>
     </row>
     <row r="10" ht="19.5" customHeight="1">
-      <c r="A10" s="38" t="s">
-        <v>173</v>
-      </c>
-      <c r="B10" s="39" t="s">
+      <c r="A10" s="41" t="s">
         <v>174</v>
       </c>
-      <c r="C10" s="41">
+      <c r="B10" s="42" t="s">
+        <v>175</v>
+      </c>
+      <c r="C10" s="44">
         <v>46177</v>
       </c>
-      <c r="D10" s="35" t="str">
-        <f>IF(ISBLANK(C10),"offen","fertig")</f>
+      <c r="D10" s="37" t="str">
+        <f t="shared" ref="D10:D19" si="3">IF(ISBLANK(C10),"offen","fertig")</f>
         <v>fertig</v>
       </c>
-      <c r="E10" s="40"/>
+      <c r="E10" s="43"/>
     </row>
     <row r="11" ht="19.5" customHeight="1">
       <c r="A11" s="8" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>176</v>
-      </c>
-      <c r="C11" s="33"/>
-      <c r="D11" s="35" t="str">
-        <f>IF(ISBLANK(C11),"offen","fertig")</f>
+        <v>177</v>
+      </c>
+      <c r="C11" s="35"/>
+      <c r="D11" s="37" t="str">
+        <f t="shared" si="3"/>
         <v>offen</v>
       </c>
-      <c r="E11" s="40"/>
+      <c r="E11" s="43"/>
     </row>
     <row r="12" ht="19.5" customHeight="1">
-      <c r="A12" s="38" t="s">
-        <v>177</v>
-      </c>
-      <c r="B12" s="39" t="s">
+      <c r="A12" s="41" t="s">
         <v>178</v>
       </c>
-      <c r="C12" s="33"/>
-      <c r="D12" s="35" t="str">
-        <f>IF(ISBLANK(C12),"offen","fertig")</f>
+      <c r="B12" s="42" t="s">
+        <v>179</v>
+      </c>
+      <c r="C12" s="35"/>
+      <c r="D12" s="37" t="str">
+        <f t="shared" si="3"/>
         <v>offen</v>
       </c>
-      <c r="E12" s="40"/>
+      <c r="E12" s="43"/>
     </row>
     <row r="13" ht="19.5" customHeight="1">
       <c r="A13" s="8" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>180</v>
-      </c>
-      <c r="C13" s="33"/>
-      <c r="D13" s="35" t="str">
-        <f>IF(ISBLANK(C13),"offen","fertig")</f>
+        <v>181</v>
+      </c>
+      <c r="C13" s="35"/>
+      <c r="D13" s="37" t="str">
+        <f t="shared" si="3"/>
         <v>offen</v>
       </c>
-      <c r="E13" s="40"/>
+      <c r="E13" s="43"/>
     </row>
     <row r="14" ht="19.5" customHeight="1">
-      <c r="A14" s="38" t="s">
-        <v>181</v>
-      </c>
-      <c r="B14" s="39" t="s">
+      <c r="A14" s="41" t="s">
         <v>182</v>
       </c>
-      <c r="C14" s="33"/>
-      <c r="D14" s="35" t="str">
-        <f>IF(ISBLANK(C14),"offen","fertig")</f>
+      <c r="B14" s="42" t="s">
+        <v>183</v>
+      </c>
+      <c r="C14" s="35"/>
+      <c r="D14" s="37" t="str">
+        <f t="shared" si="3"/>
         <v>offen</v>
       </c>
-      <c r="E14" s="40"/>
+      <c r="E14" s="43"/>
     </row>
     <row r="15" ht="19.5" customHeight="1">
       <c r="A15" s="8" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>184</v>
-      </c>
-      <c r="C15" s="33"/>
-      <c r="D15" s="35" t="str">
-        <f>IF(ISBLANK(C15),"offen","fertig")</f>
+        <v>185</v>
+      </c>
+      <c r="C15" s="35"/>
+      <c r="D15" s="37" t="str">
+        <f t="shared" si="3"/>
         <v>offen</v>
       </c>
-      <c r="E15" s="40"/>
+      <c r="E15" s="43"/>
     </row>
     <row r="16" ht="19.5" customHeight="1">
-      <c r="A16" s="38" t="s">
-        <v>185</v>
-      </c>
-      <c r="B16" s="39" t="s">
+      <c r="A16" s="41" t="s">
         <v>186</v>
       </c>
-      <c r="C16" s="33"/>
-      <c r="D16" s="35" t="str">
-        <f>IF(ISBLANK(C16),"offen","fertig")</f>
+      <c r="B16" s="42" t="s">
+        <v>187</v>
+      </c>
+      <c r="C16" s="35"/>
+      <c r="D16" s="37" t="str">
+        <f t="shared" si="3"/>
         <v>offen</v>
       </c>
-      <c r="E16" s="40"/>
+      <c r="E16" s="43"/>
     </row>
     <row r="17" ht="19.5" customHeight="1">
       <c r="A17" s="8" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>188</v>
-      </c>
-      <c r="C17" s="33"/>
-      <c r="D17" s="35" t="str">
-        <f>IF(ISBLANK(C17),"offen","fertig")</f>
+        <v>189</v>
+      </c>
+      <c r="C17" s="35"/>
+      <c r="D17" s="37" t="str">
+        <f t="shared" si="3"/>
         <v>offen</v>
       </c>
-      <c r="E17" s="40"/>
+      <c r="E17" s="43"/>
     </row>
     <row r="18" ht="19.5" customHeight="1">
-      <c r="A18" s="38" t="s">
-        <v>189</v>
-      </c>
-      <c r="B18" s="39" t="s">
+      <c r="A18" s="41" t="s">
         <v>190</v>
       </c>
-      <c r="C18" s="33"/>
-      <c r="D18" s="35" t="str">
-        <f>IF(ISBLANK(C18),"offen","fertig")</f>
+      <c r="B18" s="42" t="s">
+        <v>191</v>
+      </c>
+      <c r="C18" s="35"/>
+      <c r="D18" s="37" t="str">
+        <f t="shared" si="3"/>
         <v>offen</v>
       </c>
-      <c r="E18" s="40"/>
+      <c r="E18" s="43"/>
     </row>
     <row r="19" ht="19.5" customHeight="1">
       <c r="A19" s="8" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>192</v>
-      </c>
-      <c r="C19" s="33"/>
-      <c r="D19" s="35" t="str">
-        <f>IF(ISBLANK(C19),"offen","fertig")</f>
+        <v>193</v>
+      </c>
+      <c r="C19" s="35"/>
+      <c r="D19" s="37" t="str">
+        <f t="shared" si="3"/>
         <v>offen</v>
       </c>
-      <c r="E19" s="40"/>
+      <c r="E19" s="43"/>
     </row>
     <row r="22" ht="6" customHeight="1"/>
     <row r="23" ht="15" customHeight="1">
-      <c r="A23" s="42" t="s">
-        <v>193</v>
-      </c>
-      <c r="B23" s="42"/>
-      <c r="C23" s="42"/>
-      <c r="D23" s="42"/>
-      <c r="E23" s="42"/>
+      <c r="A23" s="45" t="s">
+        <v>194</v>
+      </c>
+      <c r="B23" s="45"/>
+      <c r="C23" s="45"/>
+      <c r="D23" s="45"/>
+      <c r="E23" s="45"/>
     </row>
     <row r="24" ht="19.5" customHeight="1">
-      <c r="A24" s="43" t="s">
+      <c r="A24" s="46" t="s">
         <v>91</v>
       </c>
-      <c r="B24" s="44" t="s">
-        <v>170</v>
-      </c>
-      <c r="C24" s="44"/>
-      <c r="D24" s="44"/>
-      <c r="E24" s="44"/>
+      <c r="B24" s="47" t="s">
+        <v>171</v>
+      </c>
+      <c r="C24" s="47"/>
+      <c r="D24" s="47"/>
+      <c r="E24" s="47"/>
     </row>
     <row r="25" ht="19.5" customHeight="1">
-      <c r="A25" s="43" t="s">
+      <c r="A25" s="46" t="s">
         <v>92</v>
       </c>
-      <c r="B25" s="45"/>
-      <c r="C25" s="45"/>
-      <c r="D25" s="45"/>
-      <c r="E25" s="45"/>
+      <c r="B25" s="48"/>
+      <c r="C25" s="48"/>
+      <c r="D25" s="48"/>
+      <c r="E25" s="48"/>
     </row>
     <row r="26" ht="19.5" customHeight="1">
-      <c r="A26" s="43" t="s">
-        <v>194</v>
-      </c>
-      <c r="B26" s="45"/>
-      <c r="C26" s="45"/>
-      <c r="D26" s="45"/>
-      <c r="E26" s="45"/>
+      <c r="A26" s="46" t="s">
+        <v>195</v>
+      </c>
+      <c r="B26" s="48"/>
+      <c r="C26" s="48"/>
+      <c r="D26" s="48"/>
+      <c r="E26" s="48"/>
     </row>
     <row r="27" ht="19.5" customHeight="1">
-      <c r="A27" s="43" t="s">
+      <c r="A27" s="46" t="s">
         <v>103</v>
       </c>
-      <c r="B27" s="45" t="s">
-        <v>104</v>
-      </c>
-      <c r="C27" s="45"/>
-      <c r="D27" s="45"/>
-      <c r="E27" s="45"/>
+      <c r="B27" s="48" t="s">
+        <v>137</v>
+      </c>
+      <c r="C27" s="48"/>
+      <c r="D27" s="48"/>
+      <c r="E27" s="48"/>
     </row>
     <row r="28" ht="19.5" customHeight="1">
-      <c r="A28" s="43" t="s">
+      <c r="A28" s="46" t="s">
         <v>106</v>
       </c>
-      <c r="B28" s="45"/>
-      <c r="C28" s="45"/>
-      <c r="D28" s="45"/>
-      <c r="E28" s="45"/>
+      <c r="B28" s="48"/>
+      <c r="C28" s="48"/>
+      <c r="D28" s="48"/>
+      <c r="E28" s="48"/>
     </row>
     <row r="29" ht="19.5" customHeight="1">
-      <c r="A29" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="B29" s="45"/>
-      <c r="C29" s="45"/>
-      <c r="D29" s="45"/>
-      <c r="E29" s="45"/>
+      <c r="A29" s="46" t="s">
+        <v>196</v>
+      </c>
+      <c r="B29" s="48"/>
+      <c r="C29" s="48"/>
+      <c r="D29" s="48"/>
+      <c r="E29" s="48"/>
     </row>
     <row r="30" ht="6" customHeight="1"/>
     <row r="32" ht="15" customHeight="1">
-      <c r="A32" s="42" t="s">
+      <c r="A32" s="45" t="s">
+        <v>197</v>
+      </c>
+      <c r="B32" s="45"/>
+      <c r="C32" s="45"/>
+      <c r="D32" s="45"/>
+      <c r="E32" s="45"/>
+    </row>
+    <row r="33" ht="19.5" customHeight="1">
+      <c r="A33" s="46" t="s">
+        <v>91</v>
+      </c>
+      <c r="B33" s="47" t="s">
+        <v>173</v>
+      </c>
+      <c r="C33" s="47"/>
+      <c r="D33" s="47"/>
+      <c r="E33" s="47"/>
+    </row>
+    <row r="34" ht="19.5" customHeight="1">
+      <c r="A34" s="46" t="s">
+        <v>92</v>
+      </c>
+      <c r="B34" s="48"/>
+      <c r="C34" s="48"/>
+      <c r="D34" s="48"/>
+      <c r="E34" s="48"/>
+    </row>
+    <row r="35" ht="19.5" customHeight="1">
+      <c r="A35" s="46" t="s">
+        <v>195</v>
+      </c>
+      <c r="B35" s="48"/>
+      <c r="C35" s="48"/>
+      <c r="D35" s="48"/>
+      <c r="E35" s="48"/>
+    </row>
+    <row r="36" ht="19.5" customHeight="1">
+      <c r="A36" s="46" t="s">
+        <v>103</v>
+      </c>
+      <c r="B36" s="48" t="s">
+        <v>137</v>
+      </c>
+      <c r="C36" s="48"/>
+      <c r="D36" s="48"/>
+      <c r="E36" s="48"/>
+    </row>
+    <row r="37" ht="19.5" customHeight="1">
+      <c r="A37" s="46" t="s">
+        <v>106</v>
+      </c>
+      <c r="B37" s="48"/>
+      <c r="C37" s="48"/>
+      <c r="D37" s="48"/>
+      <c r="E37" s="48"/>
+    </row>
+    <row r="38" ht="19.5" customHeight="1">
+      <c r="A38" s="46" t="s">
         <v>196</v>
       </c>
-      <c r="B32" s="42"/>
-      <c r="C32" s="42"/>
-      <c r="D32" s="42"/>
-      <c r="E32" s="42"/>
-    </row>
-    <row r="33" ht="19.5" customHeight="1">
-      <c r="A33" s="43" t="s">
-        <v>91</v>
-      </c>
-      <c r="B33" s="44" t="s">
-        <v>172</v>
-      </c>
-      <c r="C33" s="44"/>
-      <c r="D33" s="44"/>
-      <c r="E33" s="44"/>
-    </row>
-    <row r="34" ht="19.5" customHeight="1">
-      <c r="A34" s="43" t="s">
-        <v>92</v>
-      </c>
-      <c r="B34" s="45"/>
-      <c r="C34" s="45"/>
-      <c r="D34" s="45"/>
-      <c r="E34" s="45"/>
-    </row>
-    <row r="35" ht="19.5" customHeight="1">
-      <c r="A35" s="43" t="s">
-        <v>194</v>
-      </c>
-      <c r="B35" s="45"/>
-      <c r="C35" s="45"/>
-      <c r="D35" s="45"/>
-      <c r="E35" s="45"/>
-    </row>
-    <row r="36" ht="19.5" customHeight="1">
-      <c r="A36" s="43" t="s">
-        <v>103</v>
-      </c>
-      <c r="B36" s="45" t="s">
-        <v>104</v>
-      </c>
-      <c r="C36" s="45"/>
-      <c r="D36" s="45"/>
-      <c r="E36" s="45"/>
-    </row>
-    <row r="37" ht="19.5" customHeight="1">
-      <c r="A37" s="43" t="s">
-        <v>106</v>
-      </c>
-      <c r="B37" s="45"/>
-      <c r="C37" s="45"/>
-      <c r="D37" s="45"/>
-      <c r="E37" s="45"/>
-    </row>
-    <row r="38" ht="19.5" customHeight="1">
-      <c r="A38" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="B38" s="45"/>
-      <c r="C38" s="45"/>
-      <c r="D38" s="45"/>
-      <c r="E38" s="45"/>
+      <c r="B38" s="48"/>
+      <c r="C38" s="48"/>
+      <c r="D38" s="48"/>
+      <c r="E38" s="48"/>
     </row>
     <row r="39" ht="6" customHeight="1"/>
     <row r="41" ht="15" customHeight="1">
-      <c r="A41" s="42" t="s">
-        <v>197</v>
-      </c>
-      <c r="B41" s="42"/>
-      <c r="C41" s="42"/>
-      <c r="D41" s="42"/>
-      <c r="E41" s="42"/>
+      <c r="A41" s="45" t="s">
+        <v>198</v>
+      </c>
+      <c r="B41" s="45"/>
+      <c r="C41" s="45"/>
+      <c r="D41" s="45"/>
+      <c r="E41" s="45"/>
     </row>
     <row r="42" ht="19.5" customHeight="1">
-      <c r="A42" s="43" t="s">
+      <c r="A42" s="46" t="s">
         <v>91</v>
       </c>
-      <c r="B42" s="44" t="s">
-        <v>174</v>
-      </c>
-      <c r="C42" s="44"/>
-      <c r="D42" s="44"/>
-      <c r="E42" s="44"/>
+      <c r="B42" s="47" t="s">
+        <v>175</v>
+      </c>
+      <c r="C42" s="47"/>
+      <c r="D42" s="47"/>
+      <c r="E42" s="47"/>
     </row>
     <row r="43" ht="19.5" customHeight="1">
-      <c r="A43" s="43" t="s">
+      <c r="A43" s="46" t="s">
         <v>92</v>
       </c>
-      <c r="B43" s="45"/>
-      <c r="C43" s="45"/>
-      <c r="D43" s="45"/>
-      <c r="E43" s="45"/>
+      <c r="B43" s="48"/>
+      <c r="C43" s="48"/>
+      <c r="D43" s="48"/>
+      <c r="E43" s="48"/>
     </row>
     <row r="44" ht="19.5" customHeight="1">
-      <c r="A44" s="43" t="s">
-        <v>194</v>
-      </c>
-      <c r="B44" s="45"/>
-      <c r="C44" s="45"/>
-      <c r="D44" s="45"/>
-      <c r="E44" s="45"/>
+      <c r="A44" s="46" t="s">
+        <v>195</v>
+      </c>
+      <c r="B44" s="48"/>
+      <c r="C44" s="48"/>
+      <c r="D44" s="48"/>
+      <c r="E44" s="48"/>
     </row>
     <row r="45" ht="19.5" customHeight="1">
-      <c r="A45" s="43" t="s">
+      <c r="A45" s="46" t="s">
         <v>103</v>
       </c>
-      <c r="B45" s="45" t="s">
-        <v>104</v>
-      </c>
-      <c r="C45" s="45"/>
-      <c r="D45" s="45"/>
-      <c r="E45" s="45"/>
+      <c r="B45" s="48" t="s">
+        <v>137</v>
+      </c>
+      <c r="C45" s="48"/>
+      <c r="D45" s="48"/>
+      <c r="E45" s="48"/>
     </row>
     <row r="46" ht="19.5" customHeight="1">
-      <c r="A46" s="43" t="s">
+      <c r="A46" s="46" t="s">
         <v>106</v>
       </c>
-      <c r="B46" s="45"/>
-      <c r="C46" s="45"/>
-      <c r="D46" s="45"/>
-      <c r="E46" s="45"/>
+      <c r="B46" s="48"/>
+      <c r="C46" s="48"/>
+      <c r="D46" s="48"/>
+      <c r="E46" s="48"/>
     </row>
     <row r="47" ht="19.5" customHeight="1">
-      <c r="A47" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="B47" s="45"/>
-      <c r="C47" s="45"/>
-      <c r="D47" s="45"/>
-      <c r="E47" s="45"/>
+      <c r="A47" s="46" t="s">
+        <v>196</v>
+      </c>
+      <c r="B47" s="48"/>
+      <c r="C47" s="48"/>
+      <c r="D47" s="48"/>
+      <c r="E47" s="48"/>
     </row>
     <row r="48" ht="6" customHeight="1"/>
     <row r="50" ht="15" customHeight="1">
-      <c r="A50" s="42" t="s">
-        <v>198</v>
-      </c>
-      <c r="B50" s="42"/>
-      <c r="C50" s="42"/>
-      <c r="D50" s="42"/>
-      <c r="E50" s="42"/>
+      <c r="A50" s="45" t="s">
+        <v>199</v>
+      </c>
+      <c r="B50" s="45"/>
+      <c r="C50" s="45"/>
+      <c r="D50" s="45"/>
+      <c r="E50" s="45"/>
     </row>
     <row r="51" ht="19.5" customHeight="1">
-      <c r="A51" s="43" t="s">
+      <c r="A51" s="46" t="s">
         <v>91</v>
       </c>
-      <c r="B51" s="44" t="s">
-        <v>176</v>
-      </c>
-      <c r="C51" s="44"/>
-      <c r="D51" s="44"/>
-      <c r="E51" s="44"/>
+      <c r="B51" s="47" t="s">
+        <v>177</v>
+      </c>
+      <c r="C51" s="47"/>
+      <c r="D51" s="47"/>
+      <c r="E51" s="47"/>
     </row>
     <row r="52" ht="19.5" customHeight="1">
-      <c r="A52" s="43" t="s">
+      <c r="A52" s="46" t="s">
         <v>92</v>
       </c>
-      <c r="B52" s="45"/>
-      <c r="C52" s="45"/>
-      <c r="D52" s="45"/>
-      <c r="E52" s="45"/>
+      <c r="B52" s="48"/>
+      <c r="C52" s="48"/>
+      <c r="D52" s="48"/>
+      <c r="E52" s="48"/>
     </row>
     <row r="53" ht="19.5" customHeight="1">
-      <c r="A53" s="43" t="s">
-        <v>194</v>
-      </c>
-      <c r="B53" s="45"/>
-      <c r="C53" s="45"/>
-      <c r="D53" s="45"/>
-      <c r="E53" s="45"/>
+      <c r="A53" s="46" t="s">
+        <v>195</v>
+      </c>
+      <c r="B53" s="48"/>
+      <c r="C53" s="48"/>
+      <c r="D53" s="48"/>
+      <c r="E53" s="48"/>
     </row>
     <row r="54" ht="19.5" customHeight="1">
-      <c r="A54" s="43" t="s">
+      <c r="A54" s="46" t="s">
         <v>103</v>
       </c>
-      <c r="B54" s="45" t="s">
-        <v>104</v>
-      </c>
-      <c r="C54" s="45"/>
-      <c r="D54" s="45"/>
-      <c r="E54" s="45"/>
+      <c r="B54" s="48" t="s">
+        <v>137</v>
+      </c>
+      <c r="C54" s="48"/>
+      <c r="D54" s="48"/>
+      <c r="E54" s="48"/>
     </row>
     <row r="55" ht="19.5" customHeight="1">
-      <c r="A55" s="43" t="s">
+      <c r="A55" s="46" t="s">
         <v>106</v>
       </c>
-      <c r="B55" s="45"/>
-      <c r="C55" s="45"/>
-      <c r="D55" s="45"/>
-      <c r="E55" s="45"/>
+      <c r="B55" s="48"/>
+      <c r="C55" s="48"/>
+      <c r="D55" s="48"/>
+      <c r="E55" s="48"/>
     </row>
     <row r="56" ht="19.5" customHeight="1">
-      <c r="A56" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="B56" s="45"/>
-      <c r="C56" s="45"/>
-      <c r="D56" s="45"/>
-      <c r="E56" s="45"/>
+      <c r="A56" s="46" t="s">
+        <v>196</v>
+      </c>
+      <c r="B56" s="48"/>
+      <c r="C56" s="48"/>
+      <c r="D56" s="48"/>
+      <c r="E56" s="48"/>
     </row>
     <row r="57" ht="6" customHeight="1"/>
     <row r="59" ht="15" customHeight="1">
-      <c r="A59" s="42" t="s">
-        <v>199</v>
-      </c>
-      <c r="B59" s="42"/>
-      <c r="C59" s="42"/>
-      <c r="D59" s="42"/>
-      <c r="E59" s="42"/>
+      <c r="A59" s="45" t="s">
+        <v>200</v>
+      </c>
+      <c r="B59" s="45"/>
+      <c r="C59" s="45"/>
+      <c r="D59" s="45"/>
+      <c r="E59" s="45"/>
     </row>
     <row r="60" ht="19.5" customHeight="1">
-      <c r="A60" s="43" t="s">
+      <c r="A60" s="46" t="s">
         <v>91</v>
       </c>
-      <c r="B60" s="44" t="s">
-        <v>178</v>
-      </c>
-      <c r="C60" s="44"/>
-      <c r="D60" s="44"/>
-      <c r="E60" s="44"/>
+      <c r="B60" s="47" t="s">
+        <v>179</v>
+      </c>
+      <c r="C60" s="47"/>
+      <c r="D60" s="47"/>
+      <c r="E60" s="47"/>
     </row>
     <row r="61" ht="19.5" customHeight="1">
-      <c r="A61" s="43" t="s">
+      <c r="A61" s="46" t="s">
         <v>92</v>
       </c>
-      <c r="B61" s="45"/>
-      <c r="C61" s="45"/>
-      <c r="D61" s="45"/>
-      <c r="E61" s="45"/>
+      <c r="B61" s="48"/>
+      <c r="C61" s="48"/>
+      <c r="D61" s="48"/>
+      <c r="E61" s="48"/>
     </row>
     <row r="62" ht="19.5" customHeight="1">
-      <c r="A62" s="43" t="s">
-        <v>194</v>
-      </c>
-      <c r="B62" s="45"/>
-      <c r="C62" s="45"/>
-      <c r="D62" s="45"/>
-      <c r="E62" s="45"/>
+      <c r="A62" s="46" t="s">
+        <v>195</v>
+      </c>
+      <c r="B62" s="48"/>
+      <c r="C62" s="48"/>
+      <c r="D62" s="48"/>
+      <c r="E62" s="48"/>
     </row>
     <row r="63" ht="19.5" customHeight="1">
-      <c r="A63" s="43" t="s">
+      <c r="A63" s="46" t="s">
         <v>103</v>
       </c>
-      <c r="B63" s="45" t="s">
-        <v>104</v>
-      </c>
-      <c r="C63" s="45"/>
-      <c r="D63" s="45"/>
-      <c r="E63" s="45"/>
+      <c r="B63" s="48" t="s">
+        <v>137</v>
+      </c>
+      <c r="C63" s="48"/>
+      <c r="D63" s="48"/>
+      <c r="E63" s="48"/>
     </row>
     <row r="64" ht="19.5" customHeight="1">
-      <c r="A64" s="43" t="s">
+      <c r="A64" s="46" t="s">
         <v>106</v>
       </c>
-      <c r="B64" s="45"/>
-      <c r="C64" s="45"/>
-      <c r="D64" s="45"/>
-      <c r="E64" s="45"/>
+      <c r="B64" s="48"/>
+      <c r="C64" s="48"/>
+      <c r="D64" s="48"/>
+      <c r="E64" s="48"/>
     </row>
     <row r="65" ht="19.5" customHeight="1">
-      <c r="A65" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="B65" s="45"/>
-      <c r="C65" s="45"/>
-      <c r="D65" s="45"/>
-      <c r="E65" s="45"/>
+      <c r="A65" s="46" t="s">
+        <v>196</v>
+      </c>
+      <c r="B65" s="48"/>
+      <c r="C65" s="48"/>
+      <c r="D65" s="48"/>
+      <c r="E65" s="48"/>
     </row>
     <row r="66" ht="6" customHeight="1"/>
     <row r="68" ht="15" customHeight="1">
-      <c r="A68" s="42" t="s">
-        <v>200</v>
-      </c>
-      <c r="B68" s="42"/>
-      <c r="C68" s="42"/>
-      <c r="D68" s="42"/>
-      <c r="E68" s="42"/>
+      <c r="A68" s="45" t="s">
+        <v>201</v>
+      </c>
+      <c r="B68" s="45"/>
+      <c r="C68" s="45"/>
+      <c r="D68" s="45"/>
+      <c r="E68" s="45"/>
     </row>
     <row r="69" ht="19.5" customHeight="1">
-      <c r="A69" s="43" t="s">
+      <c r="A69" s="46" t="s">
         <v>91</v>
       </c>
-      <c r="B69" s="44" t="s">
-        <v>180</v>
-      </c>
-      <c r="C69" s="44"/>
-      <c r="D69" s="44"/>
-      <c r="E69" s="44"/>
+      <c r="B69" s="47" t="s">
+        <v>181</v>
+      </c>
+      <c r="C69" s="47"/>
+      <c r="D69" s="47"/>
+      <c r="E69" s="47"/>
     </row>
     <row r="70" ht="19.5" customHeight="1">
-      <c r="A70" s="43" t="s">
+      <c r="A70" s="46" t="s">
         <v>92</v>
       </c>
-      <c r="B70" s="45"/>
-      <c r="C70" s="45"/>
-      <c r="D70" s="45"/>
-      <c r="E70" s="45"/>
+      <c r="B70" s="48"/>
+      <c r="C70" s="48"/>
+      <c r="D70" s="48"/>
+      <c r="E70" s="48"/>
     </row>
     <row r="71" ht="19.5" customHeight="1">
-      <c r="A71" s="43" t="s">
-        <v>194</v>
-      </c>
-      <c r="B71" s="45"/>
-      <c r="C71" s="45"/>
-      <c r="D71" s="45"/>
-      <c r="E71" s="45"/>
+      <c r="A71" s="46" t="s">
+        <v>195</v>
+      </c>
+      <c r="B71" s="48"/>
+      <c r="C71" s="48"/>
+      <c r="D71" s="48"/>
+      <c r="E71" s="48"/>
     </row>
     <row r="72" ht="19.5" customHeight="1">
-      <c r="A72" s="43" t="s">
+      <c r="A72" s="46" t="s">
         <v>103</v>
       </c>
-      <c r="B72" s="45" t="s">
-        <v>104</v>
-      </c>
-      <c r="C72" s="45"/>
-      <c r="D72" s="45"/>
-      <c r="E72" s="45"/>
+      <c r="B72" s="48" t="s">
+        <v>137</v>
+      </c>
+      <c r="C72" s="48"/>
+      <c r="D72" s="48"/>
+      <c r="E72" s="48"/>
     </row>
     <row r="73" ht="19.5" customHeight="1">
-      <c r="A73" s="43" t="s">
+      <c r="A73" s="46" t="s">
         <v>106</v>
       </c>
-      <c r="B73" s="45"/>
-      <c r="C73" s="45"/>
-      <c r="D73" s="45"/>
-      <c r="E73" s="45"/>
+      <c r="B73" s="48"/>
+      <c r="C73" s="48"/>
+      <c r="D73" s="48"/>
+      <c r="E73" s="48"/>
     </row>
     <row r="74" ht="19.5" customHeight="1">
-      <c r="A74" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="B74" s="45"/>
-      <c r="C74" s="45"/>
-      <c r="D74" s="45"/>
-      <c r="E74" s="45"/>
+      <c r="A74" s="46" t="s">
+        <v>196</v>
+      </c>
+      <c r="B74" s="48"/>
+      <c r="C74" s="48"/>
+      <c r="D74" s="48"/>
+      <c r="E74" s="48"/>
     </row>
     <row r="75" ht="6" customHeight="1"/>
     <row r="77" ht="15" customHeight="1">
-      <c r="A77" s="42" t="s">
-        <v>201</v>
-      </c>
-      <c r="B77" s="42"/>
-      <c r="C77" s="42"/>
-      <c r="D77" s="42"/>
-      <c r="E77" s="42"/>
+      <c r="A77" s="45" t="s">
+        <v>202</v>
+      </c>
+      <c r="B77" s="45"/>
+      <c r="C77" s="45"/>
+      <c r="D77" s="45"/>
+      <c r="E77" s="45"/>
     </row>
     <row r="78" ht="19.5" customHeight="1">
-      <c r="A78" s="43" t="s">
+      <c r="A78" s="46" t="s">
         <v>91</v>
       </c>
-      <c r="B78" s="44" t="s">
-        <v>182</v>
-      </c>
-      <c r="C78" s="44"/>
-      <c r="D78" s="44"/>
-      <c r="E78" s="44"/>
+      <c r="B78" s="47" t="s">
+        <v>183</v>
+      </c>
+      <c r="C78" s="47"/>
+      <c r="D78" s="47"/>
+      <c r="E78" s="47"/>
     </row>
     <row r="79" ht="19.5" customHeight="1">
-      <c r="A79" s="43" t="s">
+      <c r="A79" s="46" t="s">
         <v>92</v>
       </c>
-      <c r="B79" s="45"/>
-      <c r="C79" s="45"/>
-      <c r="D79" s="45"/>
-      <c r="E79" s="45"/>
+      <c r="B79" s="48"/>
+      <c r="C79" s="48"/>
+      <c r="D79" s="48"/>
+      <c r="E79" s="48"/>
     </row>
     <row r="80" ht="19.5" customHeight="1">
-      <c r="A80" s="43" t="s">
-        <v>194</v>
-      </c>
-      <c r="B80" s="45"/>
-      <c r="C80" s="45"/>
-      <c r="D80" s="45"/>
-      <c r="E80" s="45"/>
+      <c r="A80" s="46" t="s">
+        <v>195</v>
+      </c>
+      <c r="B80" s="48"/>
+      <c r="C80" s="48"/>
+      <c r="D80" s="48"/>
+      <c r="E80" s="48"/>
     </row>
     <row r="81" ht="19.5" customHeight="1">
-      <c r="A81" s="43" t="s">
+      <c r="A81" s="46" t="s">
         <v>103</v>
       </c>
-      <c r="B81" s="45" t="s">
-        <v>104</v>
-      </c>
-      <c r="C81" s="45"/>
-      <c r="D81" s="45"/>
-      <c r="E81" s="45"/>
+      <c r="B81" s="48" t="s">
+        <v>137</v>
+      </c>
+      <c r="C81" s="48"/>
+      <c r="D81" s="48"/>
+      <c r="E81" s="48"/>
     </row>
     <row r="82" ht="19.5" customHeight="1">
-      <c r="A82" s="43" t="s">
+      <c r="A82" s="46" t="s">
         <v>106</v>
       </c>
-      <c r="B82" s="45"/>
-      <c r="C82" s="45"/>
-      <c r="D82" s="45"/>
-      <c r="E82" s="45"/>
+      <c r="B82" s="48"/>
+      <c r="C82" s="48"/>
+      <c r="D82" s="48"/>
+      <c r="E82" s="48"/>
     </row>
     <row r="83" ht="19.5" customHeight="1">
-      <c r="A83" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="B83" s="45"/>
-      <c r="C83" s="45"/>
-      <c r="D83" s="45"/>
-      <c r="E83" s="45"/>
+      <c r="A83" s="46" t="s">
+        <v>196</v>
+      </c>
+      <c r="B83" s="48"/>
+      <c r="C83" s="48"/>
+      <c r="D83" s="48"/>
+      <c r="E83" s="48"/>
     </row>
     <row r="84" ht="6" customHeight="1"/>
     <row r="86" ht="15" customHeight="1">
-      <c r="A86" s="42" t="s">
-        <v>202</v>
-      </c>
-      <c r="B86" s="42"/>
-      <c r="C86" s="42"/>
-      <c r="D86" s="42"/>
-      <c r="E86" s="42"/>
+      <c r="A86" s="45" t="s">
+        <v>203</v>
+      </c>
+      <c r="B86" s="45"/>
+      <c r="C86" s="45"/>
+      <c r="D86" s="45"/>
+      <c r="E86" s="45"/>
     </row>
     <row r="87" ht="19.5" customHeight="1">
-      <c r="A87" s="43" t="s">
+      <c r="A87" s="46" t="s">
         <v>91</v>
       </c>
-      <c r="B87" s="44" t="s">
-        <v>184</v>
-      </c>
-      <c r="C87" s="44"/>
-      <c r="D87" s="44"/>
-      <c r="E87" s="44"/>
+      <c r="B87" s="47" t="s">
+        <v>185</v>
+      </c>
+      <c r="C87" s="47"/>
+      <c r="D87" s="47"/>
+      <c r="E87" s="47"/>
     </row>
     <row r="88" ht="19.5" customHeight="1">
-      <c r="A88" s="43" t="s">
+      <c r="A88" s="46" t="s">
         <v>92</v>
       </c>
-      <c r="B88" s="45"/>
-      <c r="C88" s="45"/>
-      <c r="D88" s="45"/>
-      <c r="E88" s="45"/>
+      <c r="B88" s="48"/>
+      <c r="C88" s="48"/>
+      <c r="D88" s="48"/>
+      <c r="E88" s="48"/>
     </row>
     <row r="89" ht="19.5" customHeight="1">
-      <c r="A89" s="43" t="s">
-        <v>194</v>
-      </c>
-      <c r="B89" s="45"/>
-      <c r="C89" s="45"/>
-      <c r="D89" s="45"/>
-      <c r="E89" s="45"/>
+      <c r="A89" s="46" t="s">
+        <v>195</v>
+      </c>
+      <c r="B89" s="48"/>
+      <c r="C89" s="48"/>
+      <c r="D89" s="48"/>
+      <c r="E89" s="48"/>
     </row>
     <row r="90" ht="19.5" customHeight="1">
-      <c r="A90" s="43" t="s">
+      <c r="A90" s="46" t="s">
         <v>103</v>
       </c>
-      <c r="B90" s="45" t="s">
-        <v>104</v>
-      </c>
-      <c r="C90" s="45"/>
-      <c r="D90" s="45"/>
-      <c r="E90" s="45"/>
+      <c r="B90" s="48" t="s">
+        <v>137</v>
+      </c>
+      <c r="C90" s="48"/>
+      <c r="D90" s="48"/>
+      <c r="E90" s="48"/>
     </row>
     <row r="91" ht="19.5" customHeight="1">
-      <c r="A91" s="43" t="s">
+      <c r="A91" s="46" t="s">
         <v>106</v>
       </c>
-      <c r="B91" s="45"/>
-      <c r="C91" s="45"/>
-      <c r="D91" s="45"/>
-      <c r="E91" s="45"/>
+      <c r="B91" s="48"/>
+      <c r="C91" s="48"/>
+      <c r="D91" s="48"/>
+      <c r="E91" s="48"/>
     </row>
     <row r="92" ht="19.5" customHeight="1">
-      <c r="A92" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="B92" s="45"/>
-      <c r="C92" s="45"/>
-      <c r="D92" s="45"/>
-      <c r="E92" s="45"/>
+      <c r="A92" s="46" t="s">
+        <v>196</v>
+      </c>
+      <c r="B92" s="48"/>
+      <c r="C92" s="48"/>
+      <c r="D92" s="48"/>
+      <c r="E92" s="48"/>
     </row>
     <row r="93" ht="6" customHeight="1"/>
     <row r="95" ht="15" customHeight="1">
-      <c r="A95" s="42" t="s">
-        <v>203</v>
-      </c>
-      <c r="B95" s="42"/>
-      <c r="C95" s="42"/>
-      <c r="D95" s="42"/>
-      <c r="E95" s="42"/>
+      <c r="A95" s="45" t="s">
+        <v>204</v>
+      </c>
+      <c r="B95" s="45"/>
+      <c r="C95" s="45"/>
+      <c r="D95" s="45"/>
+      <c r="E95" s="45"/>
     </row>
     <row r="96" ht="19.5" customHeight="1">
-      <c r="A96" s="43" t="s">
+      <c r="A96" s="46" t="s">
         <v>91</v>
       </c>
-      <c r="B96" s="44" t="s">
-        <v>186</v>
-      </c>
-      <c r="C96" s="44"/>
-      <c r="D96" s="44"/>
-      <c r="E96" s="44"/>
+      <c r="B96" s="47" t="s">
+        <v>187</v>
+      </c>
+      <c r="C96" s="47"/>
+      <c r="D96" s="47"/>
+      <c r="E96" s="47"/>
     </row>
     <row r="97" ht="19.5" customHeight="1">
-      <c r="A97" s="43" t="s">
+      <c r="A97" s="46" t="s">
         <v>92</v>
       </c>
-      <c r="B97" s="45"/>
-      <c r="C97" s="45"/>
-      <c r="D97" s="45"/>
-      <c r="E97" s="45"/>
+      <c r="B97" s="48"/>
+      <c r="C97" s="48"/>
+      <c r="D97" s="48"/>
+      <c r="E97" s="48"/>
     </row>
     <row r="98" ht="19.5" customHeight="1">
-      <c r="A98" s="43" t="s">
-        <v>194</v>
-      </c>
-      <c r="B98" s="45"/>
-      <c r="C98" s="45"/>
-      <c r="D98" s="45"/>
-      <c r="E98" s="45"/>
+      <c r="A98" s="46" t="s">
+        <v>195</v>
+      </c>
+      <c r="B98" s="48"/>
+      <c r="C98" s="48"/>
+      <c r="D98" s="48"/>
+      <c r="E98" s="48"/>
     </row>
     <row r="99" ht="19.5" customHeight="1">
-      <c r="A99" s="43" t="s">
+      <c r="A99" s="46" t="s">
         <v>103</v>
       </c>
-      <c r="B99" s="45" t="s">
-        <v>104</v>
-      </c>
-      <c r="C99" s="45"/>
-      <c r="D99" s="45"/>
-      <c r="E99" s="45"/>
+      <c r="B99" s="48" t="s">
+        <v>137</v>
+      </c>
+      <c r="C99" s="48"/>
+      <c r="D99" s="48"/>
+      <c r="E99" s="48"/>
     </row>
     <row r="100" ht="19.5" customHeight="1">
-      <c r="A100" s="43" t="s">
+      <c r="A100" s="46" t="s">
         <v>106</v>
       </c>
-      <c r="B100" s="45"/>
-      <c r="C100" s="45"/>
-      <c r="D100" s="45"/>
-      <c r="E100" s="45"/>
+      <c r="B100" s="48"/>
+      <c r="C100" s="48"/>
+      <c r="D100" s="48"/>
+      <c r="E100" s="48"/>
     </row>
     <row r="101" ht="19.5" customHeight="1">
-      <c r="A101" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="B101" s="45"/>
-      <c r="C101" s="45"/>
-      <c r="D101" s="45"/>
-      <c r="E101" s="45"/>
+      <c r="A101" s="46" t="s">
+        <v>196</v>
+      </c>
+      <c r="B101" s="48"/>
+      <c r="C101" s="48"/>
+      <c r="D101" s="48"/>
+      <c r="E101" s="48"/>
     </row>
     <row r="102" ht="6" customHeight="1"/>
     <row r="104" ht="15" customHeight="1">
-      <c r="A104" s="42" t="s">
-        <v>204</v>
-      </c>
-      <c r="B104" s="42"/>
-      <c r="C104" s="42"/>
-      <c r="D104" s="42"/>
-      <c r="E104" s="42"/>
+      <c r="A104" s="45" t="s">
+        <v>205</v>
+      </c>
+      <c r="B104" s="45"/>
+      <c r="C104" s="45"/>
+      <c r="D104" s="45"/>
+      <c r="E104" s="45"/>
     </row>
     <row r="105" ht="19.5" customHeight="1">
-      <c r="A105" s="43" t="s">
+      <c r="A105" s="46" t="s">
         <v>91</v>
       </c>
-      <c r="B105" s="44" t="s">
-        <v>188</v>
-      </c>
-      <c r="C105" s="44"/>
-      <c r="D105" s="44"/>
-      <c r="E105" s="44"/>
+      <c r="B105" s="47" t="s">
+        <v>189</v>
+      </c>
+      <c r="C105" s="47"/>
+      <c r="D105" s="47"/>
+      <c r="E105" s="47"/>
     </row>
     <row r="106" ht="19.5" customHeight="1">
-      <c r="A106" s="43" t="s">
+      <c r="A106" s="46" t="s">
         <v>92</v>
       </c>
-      <c r="B106" s="45"/>
-      <c r="C106" s="45"/>
-      <c r="D106" s="45"/>
-      <c r="E106" s="45"/>
+      <c r="B106" s="48"/>
+      <c r="C106" s="48"/>
+      <c r="D106" s="48"/>
+      <c r="E106" s="48"/>
     </row>
     <row r="107" ht="19.5" customHeight="1">
-      <c r="A107" s="43" t="s">
-        <v>194</v>
-      </c>
-      <c r="B107" s="45"/>
-      <c r="C107" s="45"/>
-      <c r="D107" s="45"/>
-      <c r="E107" s="45"/>
+      <c r="A107" s="46" t="s">
+        <v>195</v>
+      </c>
+      <c r="B107" s="48"/>
+      <c r="C107" s="48"/>
+      <c r="D107" s="48"/>
+      <c r="E107" s="48"/>
     </row>
     <row r="108" ht="19.5" customHeight="1">
-      <c r="A108" s="43" t="s">
+      <c r="A108" s="46" t="s">
         <v>103</v>
       </c>
-      <c r="B108" s="45" t="s">
-        <v>104</v>
-      </c>
-      <c r="C108" s="45"/>
-      <c r="D108" s="45"/>
-      <c r="E108" s="45"/>
+      <c r="B108" s="48" t="s">
+        <v>137</v>
+      </c>
+      <c r="C108" s="48"/>
+      <c r="D108" s="48"/>
+      <c r="E108" s="48"/>
     </row>
     <row r="109" ht="19.5" customHeight="1">
-      <c r="A109" s="43" t="s">
+      <c r="A109" s="46" t="s">
         <v>106</v>
       </c>
-      <c r="B109" s="45"/>
-      <c r="C109" s="45"/>
-      <c r="D109" s="45"/>
-      <c r="E109" s="45"/>
+      <c r="B109" s="48"/>
+      <c r="C109" s="48"/>
+      <c r="D109" s="48"/>
+      <c r="E109" s="48"/>
     </row>
     <row r="110" ht="19.5" customHeight="1">
-      <c r="A110" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="B110" s="45"/>
-      <c r="C110" s="45"/>
-      <c r="D110" s="45"/>
-      <c r="E110" s="45"/>
+      <c r="A110" s="46" t="s">
+        <v>196</v>
+      </c>
+      <c r="B110" s="48"/>
+      <c r="C110" s="48"/>
+      <c r="D110" s="48"/>
+      <c r="E110" s="48"/>
     </row>
     <row r="111" ht="6" customHeight="1"/>
     <row r="113" ht="15" customHeight="1">
-      <c r="A113" s="42" t="s">
-        <v>205</v>
-      </c>
-      <c r="B113" s="42"/>
-      <c r="C113" s="42"/>
-      <c r="D113" s="42"/>
-      <c r="E113" s="42"/>
+      <c r="A113" s="45" t="s">
+        <v>206</v>
+      </c>
+      <c r="B113" s="45"/>
+      <c r="C113" s="45"/>
+      <c r="D113" s="45"/>
+      <c r="E113" s="45"/>
     </row>
     <row r="114" ht="19.5" customHeight="1">
-      <c r="A114" s="43" t="s">
+      <c r="A114" s="46" t="s">
         <v>91</v>
       </c>
-      <c r="B114" s="44" t="s">
-        <v>190</v>
-      </c>
-      <c r="C114" s="44"/>
-      <c r="D114" s="44"/>
-      <c r="E114" s="44"/>
+      <c r="B114" s="47" t="s">
+        <v>191</v>
+      </c>
+      <c r="C114" s="47"/>
+      <c r="D114" s="47"/>
+      <c r="E114" s="47"/>
     </row>
     <row r="115" ht="19.5" customHeight="1">
-      <c r="A115" s="43" t="s">
+      <c r="A115" s="46" t="s">
         <v>92</v>
       </c>
-      <c r="B115" s="45"/>
-      <c r="C115" s="45"/>
-      <c r="D115" s="45"/>
-      <c r="E115" s="45"/>
+      <c r="B115" s="48"/>
+      <c r="C115" s="48"/>
+      <c r="D115" s="48"/>
+      <c r="E115" s="48"/>
     </row>
     <row r="116" ht="19.5" customHeight="1">
-      <c r="A116" s="43" t="s">
-        <v>194</v>
-      </c>
-      <c r="B116" s="45"/>
-      <c r="C116" s="45"/>
-      <c r="D116" s="45"/>
-      <c r="E116" s="45"/>
+      <c r="A116" s="46" t="s">
+        <v>195</v>
+      </c>
+      <c r="B116" s="48"/>
+      <c r="C116" s="48"/>
+      <c r="D116" s="48"/>
+      <c r="E116" s="48"/>
     </row>
     <row r="117" ht="19.5" customHeight="1">
-      <c r="A117" s="43" t="s">
+      <c r="A117" s="46" t="s">
         <v>103</v>
       </c>
-      <c r="B117" s="45" t="s">
-        <v>104</v>
-      </c>
-      <c r="C117" s="45"/>
-      <c r="D117" s="45"/>
-      <c r="E117" s="45"/>
+      <c r="B117" s="48" t="s">
+        <v>137</v>
+      </c>
+      <c r="C117" s="48"/>
+      <c r="D117" s="48"/>
+      <c r="E117" s="48"/>
     </row>
     <row r="118" ht="19.5" customHeight="1">
-      <c r="A118" s="43" t="s">
+      <c r="A118" s="46" t="s">
         <v>106</v>
       </c>
-      <c r="B118" s="45"/>
-      <c r="C118" s="45"/>
-      <c r="D118" s="45"/>
-      <c r="E118" s="45"/>
+      <c r="B118" s="48"/>
+      <c r="C118" s="48"/>
+      <c r="D118" s="48"/>
+      <c r="E118" s="48"/>
     </row>
     <row r="119" ht="19.5" customHeight="1">
-      <c r="A119" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="B119" s="45"/>
-      <c r="C119" s="45"/>
-      <c r="D119" s="45"/>
-      <c r="E119" s="45"/>
+      <c r="A119" s="46" t="s">
+        <v>196</v>
+      </c>
+      <c r="B119" s="48"/>
+      <c r="C119" s="48"/>
+      <c r="D119" s="48"/>
+      <c r="E119" s="48"/>
     </row>
     <row r="120" ht="6" customHeight="1"/>
     <row r="122" ht="15" customHeight="1">
-      <c r="A122" s="42" t="s">
-        <v>206</v>
-      </c>
-      <c r="B122" s="42"/>
-      <c r="C122" s="42"/>
-      <c r="D122" s="42"/>
-      <c r="E122" s="42"/>
+      <c r="A122" s="45" t="s">
+        <v>207</v>
+      </c>
+      <c r="B122" s="45"/>
+      <c r="C122" s="45"/>
+      <c r="D122" s="45"/>
+      <c r="E122" s="45"/>
     </row>
     <row r="123" ht="19.5" customHeight="1">
-      <c r="A123" s="43" t="s">
+      <c r="A123" s="46" t="s">
         <v>91</v>
       </c>
-      <c r="B123" s="44" t="s">
-        <v>192</v>
-      </c>
-      <c r="C123" s="44"/>
-      <c r="D123" s="44"/>
-      <c r="E123" s="44"/>
+      <c r="B123" s="47" t="s">
+        <v>193</v>
+      </c>
+      <c r="C123" s="47"/>
+      <c r="D123" s="47"/>
+      <c r="E123" s="47"/>
     </row>
     <row r="124" ht="19.5" customHeight="1">
-      <c r="A124" s="43" t="s">
+      <c r="A124" s="46" t="s">
         <v>92</v>
       </c>
-      <c r="B124" s="45"/>
-      <c r="C124" s="45"/>
-      <c r="D124" s="45"/>
-      <c r="E124" s="45"/>
+      <c r="B124" s="48"/>
+      <c r="C124" s="48"/>
+      <c r="D124" s="48"/>
+      <c r="E124" s="48"/>
     </row>
     <row r="125" ht="19.5" customHeight="1">
-      <c r="A125" s="43" t="s">
-        <v>194</v>
-      </c>
-      <c r="B125" s="45"/>
-      <c r="C125" s="45"/>
-      <c r="D125" s="45"/>
-      <c r="E125" s="45"/>
+      <c r="A125" s="46" t="s">
+        <v>195</v>
+      </c>
+      <c r="B125" s="48"/>
+      <c r="C125" s="48"/>
+      <c r="D125" s="48"/>
+      <c r="E125" s="48"/>
     </row>
     <row r="126" ht="19.5" customHeight="1">
-      <c r="A126" s="43" t="s">
+      <c r="A126" s="46" t="s">
         <v>103</v>
       </c>
-      <c r="B126" s="45" t="s">
-        <v>104</v>
-      </c>
-      <c r="C126" s="45"/>
-      <c r="D126" s="45"/>
-      <c r="E126" s="45"/>
+      <c r="B126" s="48" t="s">
+        <v>137</v>
+      </c>
+      <c r="C126" s="48"/>
+      <c r="D126" s="48"/>
+      <c r="E126" s="48"/>
     </row>
     <row r="127" ht="19.5" customHeight="1">
-      <c r="A127" s="43" t="s">
+      <c r="A127" s="46" t="s">
         <v>106</v>
       </c>
-      <c r="B127" s="45"/>
-      <c r="C127" s="45"/>
-      <c r="D127" s="45"/>
-      <c r="E127" s="45"/>
+      <c r="B127" s="48"/>
+      <c r="C127" s="48"/>
+      <c r="D127" s="48"/>
+      <c r="E127" s="48"/>
     </row>
     <row r="128" ht="19.5" customHeight="1">
-      <c r="A128" s="43" t="s">
-        <v>195</v>
-      </c>
-      <c r="B128" s="45"/>
-      <c r="C128" s="45"/>
-      <c r="D128" s="45"/>
-      <c r="E128" s="45"/>
+      <c r="A128" s="46" t="s">
+        <v>196</v>
+      </c>
+      <c r="B128" s="48"/>
+      <c r="C128" s="48"/>
+      <c r="D128" s="48"/>
+      <c r="E128" s="48"/>
     </row>
     <row r="129" ht="6" customHeight="1"/>
   </sheetData>
@@ -5017,7 +5061,7 @@
   <sheetData>
     <row r="1" ht="17.25" customHeight="1">
       <c r="A1" s="24" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B1" s="24"/>
       <c r="C1" s="24"/>
@@ -5027,42 +5071,42 @@
     </row>
     <row r="3" ht="24.75" customHeight="1">
       <c r="A3" s="5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="38">
+      <c r="A4" s="41">
         <v>1</v>
       </c>
-      <c r="B4" s="46">
+      <c r="B4" s="49">
         <v>46168</v>
       </c>
-      <c r="C4" s="39" t="s">
+      <c r="C4" s="42" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="47" t="s">
-        <v>214</v>
-      </c>
-      <c r="E4" s="39" t="s">
+      <c r="D4" s="50" t="s">
+        <v>215</v>
+      </c>
+      <c r="E4" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="39" t="str">
-        <f>IF(ISBLANK(B4),"offen","fertig")</f>
+      <c r="F4" s="42" t="str">
+        <f t="shared" ref="F4:F9" si="4">IF(ISBLANK(B4),"offen","fertig")</f>
         <v>fertig</v>
       </c>
     </row>
@@ -5070,41 +5114,41 @@
       <c r="A5" s="8">
         <v>2</v>
       </c>
-      <c r="B5" s="46">
+      <c r="B5" s="49">
         <v>46170</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>27</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="39" t="str">
-        <f>IF(ISBLANK(B5),"offen","fertig")</f>
+      <c r="F5" s="42" t="str">
+        <f t="shared" si="4"/>
         <v>fertig</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
-      <c r="A6" s="38">
+      <c r="A6" s="41">
         <v>3</v>
       </c>
-      <c r="B6" s="33">
+      <c r="B6" s="35">
         <v>46175</v>
       </c>
-      <c r="C6" s="39" t="s">
+      <c r="C6" s="42" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="47" t="s">
-        <v>216</v>
-      </c>
-      <c r="E6" s="39" t="s">
+      <c r="D6" s="50" t="s">
+        <v>217</v>
+      </c>
+      <c r="E6" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="F6" s="39" t="str">
-        <f>IF(ISBLANK(B6),"offen","fertig")</f>
+      <c r="F6" s="42" t="str">
+        <f t="shared" si="4"/>
         <v>fertig</v>
       </c>
     </row>
@@ -5112,37 +5156,39 @@
       <c r="A7" s="8">
         <v>4</v>
       </c>
-      <c r="B7" s="33"/>
+      <c r="B7" s="35">
+        <v>46184</v>
+      </c>
       <c r="C7" s="10" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="F7" s="39" t="str">
-        <f>IF(ISBLANK(B7),"offen","fertig")</f>
-        <v>offen</v>
+      <c r="F7" s="42" t="str">
+        <f t="shared" si="4"/>
+        <v>fertig</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="38">
+      <c r="A8" s="41">
         <v>5</v>
       </c>
-      <c r="B8" s="33"/>
-      <c r="C8" s="39" t="s">
-        <v>219</v>
-      </c>
-      <c r="D8" s="47" t="s">
+      <c r="B8" s="35"/>
+      <c r="C8" s="42" t="s">
         <v>220</v>
       </c>
-      <c r="E8" s="39" t="s">
+      <c r="D8" s="50" t="s">
+        <v>221</v>
+      </c>
+      <c r="E8" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="39" t="str">
-        <f>IF(ISBLANK(B8),"offen","fertig")</f>
+      <c r="F8" s="42" t="str">
+        <f t="shared" si="4"/>
         <v>offen</v>
       </c>
     </row>
@@ -5150,18 +5196,18 @@
       <c r="A9" s="8">
         <v>6</v>
       </c>
-      <c r="B9" s="33"/>
+      <c r="B9" s="35"/>
       <c r="C9" s="10" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="F9" s="39" t="str">
-        <f>IF(ISBLANK(B9),"offen","fertig")</f>
+      <c r="F9" s="42" t="str">
+        <f t="shared" si="4"/>
         <v>offen</v>
       </c>
     </row>
@@ -5184,128 +5230,128 @@
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="48" t="s">
-        <v>223</v>
+      <c r="A1" s="51" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="49"/>
+      <c r="A5" s="52"/>
     </row>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="50" t="s">
-        <v>224</v>
+      <c r="A6" s="53" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="49" t="s">
-        <v>225</v>
+      <c r="A7" s="52" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="A8" s="49" t="s">
-        <v>226</v>
+      <c r="A8" s="52" t="s">
+        <v>227</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
-      <c r="A9" s="49" t="s">
-        <v>227</v>
+      <c r="A9" s="52" t="s">
+        <v>228</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
-      <c r="A10" s="49" t="s">
-        <v>228</v>
+      <c r="A10" s="52" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="49" t="s">
-        <v>229</v>
+      <c r="A11" s="52" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
-      <c r="A12" s="49"/>
+      <c r="A12" s="52"/>
     </row>
     <row r="13" ht="15.75" customHeight="1">
-      <c r="A13" s="50" t="s">
-        <v>230</v>
+      <c r="A13" s="53" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
-      <c r="A14" s="49" t="s">
-        <v>231</v>
+      <c r="A14" s="52" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1">
-      <c r="A15" s="49" t="s">
-        <v>232</v>
+      <c r="A15" s="52" t="s">
+        <v>233</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
-      <c r="A16" s="49" t="s">
-        <v>233</v>
+      <c r="A16" s="52" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
-      <c r="A17" s="49" t="s">
-        <v>234</v>
+      <c r="A17" s="52" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
-      <c r="A18" s="49"/>
+      <c r="A18" s="52"/>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="50" t="s">
-        <v>235</v>
+      <c r="A19" s="53" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="49" t="s">
-        <v>236</v>
+      <c r="A20" s="52" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="49" t="s">
-        <v>237</v>
+      <c r="A21" s="52" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="49"/>
+      <c r="A22" s="52"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="50" t="s">
-        <v>238</v>
+      <c r="A23" s="53" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="49" t="s">
-        <v>239</v>
+      <c r="A24" s="52" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="49" t="s">
-        <v>240</v>
+      <c r="A25" s="52" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="49" t="s">
-        <v>241</v>
+      <c r="A26" s="52" t="s">
+        <v>242</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="49"/>
+      <c r="A27" s="52"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="50" t="s">
-        <v>242</v>
+      <c r="A28" s="53" t="s">
+        <v>243</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="49" t="s">
-        <v>243</v>
+      <c r="A29" s="52" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="49" t="s">
-        <v>244</v>
+      <c r="A30" s="52" t="s">
+        <v>245</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v.0.36 Add @EnableMethodSecurity Add CSRF Add MapStruct to CartMapper Add @Mapper(componentModel = "spring") to ProductMapper Add PasswordEncoder to OAuth2 Update AdminProductController Add SSL in Query in application-prod.yml Add pagination to All lists in shop's area and admin's area Update Product Card without Button Details
</commit_message>
<xml_diff>
--- a/docs/PSP_OnlineShop.xlsx
+++ b/docs/PSP_OnlineShop.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="4"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="PSP" sheetId="1" state="visible" r:id="rId1"/>
@@ -945,7 +945,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="53">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1052,9 +1052,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="3" fillId="3" borderId="1" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="8" borderId="1" numFmtId="164" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="3" fillId="10" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3485,7 +3482,7 @@
       <c r="F20" s="39">
         <v>46192</v>
       </c>
-      <c r="G20" s="40">
+      <c r="G20" s="35">
         <v>46181</v>
       </c>
       <c r="H20" s="36">
@@ -3615,14 +3612,16 @@
       <c r="F24" s="38">
         <v>46206</v>
       </c>
-      <c r="G24" s="35"/>
-      <c r="H24" s="36" t="str">
+      <c r="G24" s="35">
+        <v>46191</v>
+      </c>
+      <c r="H24" s="36">
         <f t="shared" si="0"/>
-        <v/>
+        <v>-15</v>
       </c>
       <c r="I24" s="37" t="str">
         <f t="shared" si="1"/>
-        <v>offen</v>
+        <v>fertig</v>
       </c>
       <c r="J24" s="14" t="s">
         <v>162</v>
@@ -3962,10 +3961,10 @@
       </c>
     </row>
     <row r="8" ht="19.5" customHeight="1">
-      <c r="A8" s="41" t="s">
+      <c r="A8" s="40" t="s">
         <v>170</v>
       </c>
-      <c r="B8" s="42" t="s">
+      <c r="B8" s="41" t="s">
         <v>171</v>
       </c>
       <c r="C8" s="35">
@@ -3975,7 +3974,7 @@
         <f t="shared" ref="D8:D9" si="2">IF(ISBLANK(C8),"offen","fertig")</f>
         <v>fertig</v>
       </c>
-      <c r="E8" s="43"/>
+      <c r="E8" s="42"/>
     </row>
     <row r="9" ht="19.5" customHeight="1">
       <c r="A9" s="8" t="s">
@@ -3991,23 +3990,23 @@
         <f t="shared" si="2"/>
         <v>fertig</v>
       </c>
-      <c r="E9" s="43"/>
+      <c r="E9" s="42"/>
     </row>
     <row r="10" ht="19.5" customHeight="1">
-      <c r="A10" s="41" t="s">
+      <c r="A10" s="40" t="s">
         <v>174</v>
       </c>
-      <c r="B10" s="42" t="s">
+      <c r="B10" s="41" t="s">
         <v>175</v>
       </c>
-      <c r="C10" s="44">
+      <c r="C10" s="43">
         <v>46177</v>
       </c>
       <c r="D10" s="37" t="str">
         <f t="shared" ref="D10:D19" si="3">IF(ISBLANK(C10),"offen","fertig")</f>
         <v>fertig</v>
       </c>
-      <c r="E10" s="43"/>
+      <c r="E10" s="42"/>
     </row>
     <row r="11" ht="19.5" customHeight="1">
       <c r="A11" s="8" t="s">
@@ -4021,13 +4020,13 @@
         <f t="shared" si="3"/>
         <v>offen</v>
       </c>
-      <c r="E11" s="43"/>
+      <c r="E11" s="42"/>
     </row>
     <row r="12" ht="19.5" customHeight="1">
-      <c r="A12" s="41" t="s">
+      <c r="A12" s="40" t="s">
         <v>178</v>
       </c>
-      <c r="B12" s="42" t="s">
+      <c r="B12" s="41" t="s">
         <v>179</v>
       </c>
       <c r="C12" s="35"/>
@@ -4035,7 +4034,7 @@
         <f t="shared" si="3"/>
         <v>offen</v>
       </c>
-      <c r="E12" s="43"/>
+      <c r="E12" s="42"/>
     </row>
     <row r="13" ht="19.5" customHeight="1">
       <c r="A13" s="8" t="s">
@@ -4049,13 +4048,13 @@
         <f t="shared" si="3"/>
         <v>offen</v>
       </c>
-      <c r="E13" s="43"/>
+      <c r="E13" s="42"/>
     </row>
     <row r="14" ht="19.5" customHeight="1">
-      <c r="A14" s="41" t="s">
+      <c r="A14" s="40" t="s">
         <v>182</v>
       </c>
-      <c r="B14" s="42" t="s">
+      <c r="B14" s="41" t="s">
         <v>183</v>
       </c>
       <c r="C14" s="35"/>
@@ -4063,7 +4062,7 @@
         <f t="shared" si="3"/>
         <v>offen</v>
       </c>
-      <c r="E14" s="43"/>
+      <c r="E14" s="42"/>
     </row>
     <row r="15" ht="19.5" customHeight="1">
       <c r="A15" s="8" t="s">
@@ -4077,13 +4076,13 @@
         <f t="shared" si="3"/>
         <v>offen</v>
       </c>
-      <c r="E15" s="43"/>
+      <c r="E15" s="42"/>
     </row>
     <row r="16" ht="19.5" customHeight="1">
-      <c r="A16" s="41" t="s">
+      <c r="A16" s="40" t="s">
         <v>186</v>
       </c>
-      <c r="B16" s="42" t="s">
+      <c r="B16" s="41" t="s">
         <v>187</v>
       </c>
       <c r="C16" s="35"/>
@@ -4091,7 +4090,7 @@
         <f t="shared" si="3"/>
         <v>offen</v>
       </c>
-      <c r="E16" s="43"/>
+      <c r="E16" s="42"/>
     </row>
     <row r="17" ht="19.5" customHeight="1">
       <c r="A17" s="8" t="s">
@@ -4105,13 +4104,13 @@
         <f t="shared" si="3"/>
         <v>offen</v>
       </c>
-      <c r="E17" s="43"/>
+      <c r="E17" s="42"/>
     </row>
     <row r="18" ht="19.5" customHeight="1">
-      <c r="A18" s="41" t="s">
+      <c r="A18" s="40" t="s">
         <v>190</v>
       </c>
-      <c r="B18" s="42" t="s">
+      <c r="B18" s="41" t="s">
         <v>191</v>
       </c>
       <c r="C18" s="35"/>
@@ -4119,7 +4118,7 @@
         <f t="shared" si="3"/>
         <v>offen</v>
       </c>
-      <c r="E18" s="43"/>
+      <c r="E18" s="42"/>
     </row>
     <row r="19" ht="19.5" customHeight="1">
       <c r="A19" s="8" t="s">
@@ -4133,823 +4132,823 @@
         <f t="shared" si="3"/>
         <v>offen</v>
       </c>
-      <c r="E19" s="43"/>
+      <c r="E19" s="42"/>
     </row>
     <row r="22" ht="6" customHeight="1"/>
     <row r="23" ht="15" customHeight="1">
-      <c r="A23" s="45" t="s">
+      <c r="A23" s="44" t="s">
         <v>194</v>
       </c>
-      <c r="B23" s="45"/>
-      <c r="C23" s="45"/>
-      <c r="D23" s="45"/>
-      <c r="E23" s="45"/>
+      <c r="B23" s="44"/>
+      <c r="C23" s="44"/>
+      <c r="D23" s="44"/>
+      <c r="E23" s="44"/>
     </row>
     <row r="24" ht="19.5" customHeight="1">
-      <c r="A24" s="46" t="s">
+      <c r="A24" s="45" t="s">
         <v>91</v>
       </c>
-      <c r="B24" s="47" t="s">
+      <c r="B24" s="46" t="s">
         <v>171</v>
       </c>
-      <c r="C24" s="47"/>
-      <c r="D24" s="47"/>
-      <c r="E24" s="47"/>
+      <c r="C24" s="46"/>
+      <c r="D24" s="46"/>
+      <c r="E24" s="46"/>
     </row>
     <row r="25" ht="19.5" customHeight="1">
-      <c r="A25" s="46" t="s">
+      <c r="A25" s="45" t="s">
         <v>92</v>
       </c>
-      <c r="B25" s="48"/>
-      <c r="C25" s="48"/>
-      <c r="D25" s="48"/>
-      <c r="E25" s="48"/>
+      <c r="B25" s="47"/>
+      <c r="C25" s="47"/>
+      <c r="D25" s="47"/>
+      <c r="E25" s="47"/>
     </row>
     <row r="26" ht="19.5" customHeight="1">
-      <c r="A26" s="46" t="s">
+      <c r="A26" s="45" t="s">
         <v>195</v>
       </c>
-      <c r="B26" s="48"/>
-      <c r="C26" s="48"/>
-      <c r="D26" s="48"/>
-      <c r="E26" s="48"/>
+      <c r="B26" s="47"/>
+      <c r="C26" s="47"/>
+      <c r="D26" s="47"/>
+      <c r="E26" s="47"/>
     </row>
     <row r="27" ht="19.5" customHeight="1">
-      <c r="A27" s="46" t="s">
+      <c r="A27" s="45" t="s">
         <v>103</v>
       </c>
-      <c r="B27" s="48" t="s">
+      <c r="B27" s="47" t="s">
         <v>137</v>
       </c>
-      <c r="C27" s="48"/>
-      <c r="D27" s="48"/>
-      <c r="E27" s="48"/>
+      <c r="C27" s="47"/>
+      <c r="D27" s="47"/>
+      <c r="E27" s="47"/>
     </row>
     <row r="28" ht="19.5" customHeight="1">
-      <c r="A28" s="46" t="s">
+      <c r="A28" s="45" t="s">
         <v>106</v>
       </c>
-      <c r="B28" s="48"/>
-      <c r="C28" s="48"/>
-      <c r="D28" s="48"/>
-      <c r="E28" s="48"/>
+      <c r="B28" s="47"/>
+      <c r="C28" s="47"/>
+      <c r="D28" s="47"/>
+      <c r="E28" s="47"/>
     </row>
     <row r="29" ht="19.5" customHeight="1">
-      <c r="A29" s="46" t="s">
+      <c r="A29" s="45" t="s">
         <v>196</v>
       </c>
-      <c r="B29" s="48"/>
-      <c r="C29" s="48"/>
-      <c r="D29" s="48"/>
-      <c r="E29" s="48"/>
+      <c r="B29" s="47"/>
+      <c r="C29" s="47"/>
+      <c r="D29" s="47"/>
+      <c r="E29" s="47"/>
     </row>
     <row r="30" ht="6" customHeight="1"/>
     <row r="32" ht="15" customHeight="1">
-      <c r="A32" s="45" t="s">
+      <c r="A32" s="44" t="s">
         <v>197</v>
       </c>
-      <c r="B32" s="45"/>
-      <c r="C32" s="45"/>
-      <c r="D32" s="45"/>
-      <c r="E32" s="45"/>
+      <c r="B32" s="44"/>
+      <c r="C32" s="44"/>
+      <c r="D32" s="44"/>
+      <c r="E32" s="44"/>
     </row>
     <row r="33" ht="19.5" customHeight="1">
-      <c r="A33" s="46" t="s">
+      <c r="A33" s="45" t="s">
         <v>91</v>
       </c>
-      <c r="B33" s="47" t="s">
+      <c r="B33" s="46" t="s">
         <v>173</v>
       </c>
-      <c r="C33" s="47"/>
-      <c r="D33" s="47"/>
-      <c r="E33" s="47"/>
+      <c r="C33" s="46"/>
+      <c r="D33" s="46"/>
+      <c r="E33" s="46"/>
     </row>
     <row r="34" ht="19.5" customHeight="1">
-      <c r="A34" s="46" t="s">
+      <c r="A34" s="45" t="s">
         <v>92</v>
       </c>
-      <c r="B34" s="48"/>
-      <c r="C34" s="48"/>
-      <c r="D34" s="48"/>
-      <c r="E34" s="48"/>
+      <c r="B34" s="47"/>
+      <c r="C34" s="47"/>
+      <c r="D34" s="47"/>
+      <c r="E34" s="47"/>
     </row>
     <row r="35" ht="19.5" customHeight="1">
-      <c r="A35" s="46" t="s">
+      <c r="A35" s="45" t="s">
         <v>195</v>
       </c>
-      <c r="B35" s="48"/>
-      <c r="C35" s="48"/>
-      <c r="D35" s="48"/>
-      <c r="E35" s="48"/>
+      <c r="B35" s="47"/>
+      <c r="C35" s="47"/>
+      <c r="D35" s="47"/>
+      <c r="E35" s="47"/>
     </row>
     <row r="36" ht="19.5" customHeight="1">
-      <c r="A36" s="46" t="s">
+      <c r="A36" s="45" t="s">
         <v>103</v>
       </c>
-      <c r="B36" s="48" t="s">
+      <c r="B36" s="47" t="s">
         <v>137</v>
       </c>
-      <c r="C36" s="48"/>
-      <c r="D36" s="48"/>
-      <c r="E36" s="48"/>
+      <c r="C36" s="47"/>
+      <c r="D36" s="47"/>
+      <c r="E36" s="47"/>
     </row>
     <row r="37" ht="19.5" customHeight="1">
-      <c r="A37" s="46" t="s">
+      <c r="A37" s="45" t="s">
         <v>106</v>
       </c>
-      <c r="B37" s="48"/>
-      <c r="C37" s="48"/>
-      <c r="D37" s="48"/>
-      <c r="E37" s="48"/>
+      <c r="B37" s="47"/>
+      <c r="C37" s="47"/>
+      <c r="D37" s="47"/>
+      <c r="E37" s="47"/>
     </row>
     <row r="38" ht="19.5" customHeight="1">
-      <c r="A38" s="46" t="s">
+      <c r="A38" s="45" t="s">
         <v>196</v>
       </c>
-      <c r="B38" s="48"/>
-      <c r="C38" s="48"/>
-      <c r="D38" s="48"/>
-      <c r="E38" s="48"/>
+      <c r="B38" s="47"/>
+      <c r="C38" s="47"/>
+      <c r="D38" s="47"/>
+      <c r="E38" s="47"/>
     </row>
     <row r="39" ht="6" customHeight="1"/>
     <row r="41" ht="15" customHeight="1">
-      <c r="A41" s="45" t="s">
+      <c r="A41" s="44" t="s">
         <v>198</v>
       </c>
-      <c r="B41" s="45"/>
-      <c r="C41" s="45"/>
-      <c r="D41" s="45"/>
-      <c r="E41" s="45"/>
+      <c r="B41" s="44"/>
+      <c r="C41" s="44"/>
+      <c r="D41" s="44"/>
+      <c r="E41" s="44"/>
     </row>
     <row r="42" ht="19.5" customHeight="1">
-      <c r="A42" s="46" t="s">
+      <c r="A42" s="45" t="s">
         <v>91</v>
       </c>
-      <c r="B42" s="47" t="s">
+      <c r="B42" s="46" t="s">
         <v>175</v>
       </c>
-      <c r="C42" s="47"/>
-      <c r="D42" s="47"/>
-      <c r="E42" s="47"/>
+      <c r="C42" s="46"/>
+      <c r="D42" s="46"/>
+      <c r="E42" s="46"/>
     </row>
     <row r="43" ht="19.5" customHeight="1">
-      <c r="A43" s="46" t="s">
+      <c r="A43" s="45" t="s">
         <v>92</v>
       </c>
-      <c r="B43" s="48"/>
-      <c r="C43" s="48"/>
-      <c r="D43" s="48"/>
-      <c r="E43" s="48"/>
+      <c r="B43" s="47"/>
+      <c r="C43" s="47"/>
+      <c r="D43" s="47"/>
+      <c r="E43" s="47"/>
     </row>
     <row r="44" ht="19.5" customHeight="1">
-      <c r="A44" s="46" t="s">
+      <c r="A44" s="45" t="s">
         <v>195</v>
       </c>
-      <c r="B44" s="48"/>
-      <c r="C44" s="48"/>
-      <c r="D44" s="48"/>
-      <c r="E44" s="48"/>
+      <c r="B44" s="47"/>
+      <c r="C44" s="47"/>
+      <c r="D44" s="47"/>
+      <c r="E44" s="47"/>
     </row>
     <row r="45" ht="19.5" customHeight="1">
-      <c r="A45" s="46" t="s">
+      <c r="A45" s="45" t="s">
         <v>103</v>
       </c>
-      <c r="B45" s="48" t="s">
+      <c r="B45" s="47" t="s">
         <v>137</v>
       </c>
-      <c r="C45" s="48"/>
-      <c r="D45" s="48"/>
-      <c r="E45" s="48"/>
+      <c r="C45" s="47"/>
+      <c r="D45" s="47"/>
+      <c r="E45" s="47"/>
     </row>
     <row r="46" ht="19.5" customHeight="1">
-      <c r="A46" s="46" t="s">
+      <c r="A46" s="45" t="s">
         <v>106</v>
       </c>
-      <c r="B46" s="48"/>
-      <c r="C46" s="48"/>
-      <c r="D46" s="48"/>
-      <c r="E46" s="48"/>
+      <c r="B46" s="47"/>
+      <c r="C46" s="47"/>
+      <c r="D46" s="47"/>
+      <c r="E46" s="47"/>
     </row>
     <row r="47" ht="19.5" customHeight="1">
-      <c r="A47" s="46" t="s">
+      <c r="A47" s="45" t="s">
         <v>196</v>
       </c>
-      <c r="B47" s="48"/>
-      <c r="C47" s="48"/>
-      <c r="D47" s="48"/>
-      <c r="E47" s="48"/>
+      <c r="B47" s="47"/>
+      <c r="C47" s="47"/>
+      <c r="D47" s="47"/>
+      <c r="E47" s="47"/>
     </row>
     <row r="48" ht="6" customHeight="1"/>
     <row r="50" ht="15" customHeight="1">
-      <c r="A50" s="45" t="s">
+      <c r="A50" s="44" t="s">
         <v>199</v>
       </c>
-      <c r="B50" s="45"/>
-      <c r="C50" s="45"/>
-      <c r="D50" s="45"/>
-      <c r="E50" s="45"/>
+      <c r="B50" s="44"/>
+      <c r="C50" s="44"/>
+      <c r="D50" s="44"/>
+      <c r="E50" s="44"/>
     </row>
     <row r="51" ht="19.5" customHeight="1">
-      <c r="A51" s="46" t="s">
+      <c r="A51" s="45" t="s">
         <v>91</v>
       </c>
-      <c r="B51" s="47" t="s">
+      <c r="B51" s="46" t="s">
         <v>177</v>
       </c>
-      <c r="C51" s="47"/>
-      <c r="D51" s="47"/>
-      <c r="E51" s="47"/>
+      <c r="C51" s="46"/>
+      <c r="D51" s="46"/>
+      <c r="E51" s="46"/>
     </row>
     <row r="52" ht="19.5" customHeight="1">
-      <c r="A52" s="46" t="s">
+      <c r="A52" s="45" t="s">
         <v>92</v>
       </c>
-      <c r="B52" s="48"/>
-      <c r="C52" s="48"/>
-      <c r="D52" s="48"/>
-      <c r="E52" s="48"/>
+      <c r="B52" s="47"/>
+      <c r="C52" s="47"/>
+      <c r="D52" s="47"/>
+      <c r="E52" s="47"/>
     </row>
     <row r="53" ht="19.5" customHeight="1">
-      <c r="A53" s="46" t="s">
+      <c r="A53" s="45" t="s">
         <v>195</v>
       </c>
-      <c r="B53" s="48"/>
-      <c r="C53" s="48"/>
-      <c r="D53" s="48"/>
-      <c r="E53" s="48"/>
+      <c r="B53" s="47"/>
+      <c r="C53" s="47"/>
+      <c r="D53" s="47"/>
+      <c r="E53" s="47"/>
     </row>
     <row r="54" ht="19.5" customHeight="1">
-      <c r="A54" s="46" t="s">
+      <c r="A54" s="45" t="s">
         <v>103</v>
       </c>
-      <c r="B54" s="48" t="s">
+      <c r="B54" s="47" t="s">
         <v>137</v>
       </c>
-      <c r="C54" s="48"/>
-      <c r="D54" s="48"/>
-      <c r="E54" s="48"/>
+      <c r="C54" s="47"/>
+      <c r="D54" s="47"/>
+      <c r="E54" s="47"/>
     </row>
     <row r="55" ht="19.5" customHeight="1">
-      <c r="A55" s="46" t="s">
+      <c r="A55" s="45" t="s">
         <v>106</v>
       </c>
-      <c r="B55" s="48"/>
-      <c r="C55" s="48"/>
-      <c r="D55" s="48"/>
-      <c r="E55" s="48"/>
+      <c r="B55" s="47"/>
+      <c r="C55" s="47"/>
+      <c r="D55" s="47"/>
+      <c r="E55" s="47"/>
     </row>
     <row r="56" ht="19.5" customHeight="1">
-      <c r="A56" s="46" t="s">
+      <c r="A56" s="45" t="s">
         <v>196</v>
       </c>
-      <c r="B56" s="48"/>
-      <c r="C56" s="48"/>
-      <c r="D56" s="48"/>
-      <c r="E56" s="48"/>
+      <c r="B56" s="47"/>
+      <c r="C56" s="47"/>
+      <c r="D56" s="47"/>
+      <c r="E56" s="47"/>
     </row>
     <row r="57" ht="6" customHeight="1"/>
     <row r="59" ht="15" customHeight="1">
-      <c r="A59" s="45" t="s">
+      <c r="A59" s="44" t="s">
         <v>200</v>
       </c>
-      <c r="B59" s="45"/>
-      <c r="C59" s="45"/>
-      <c r="D59" s="45"/>
-      <c r="E59" s="45"/>
+      <c r="B59" s="44"/>
+      <c r="C59" s="44"/>
+      <c r="D59" s="44"/>
+      <c r="E59" s="44"/>
     </row>
     <row r="60" ht="19.5" customHeight="1">
-      <c r="A60" s="46" t="s">
+      <c r="A60" s="45" t="s">
         <v>91</v>
       </c>
-      <c r="B60" s="47" t="s">
+      <c r="B60" s="46" t="s">
         <v>179</v>
       </c>
-      <c r="C60" s="47"/>
-      <c r="D60" s="47"/>
-      <c r="E60" s="47"/>
+      <c r="C60" s="46"/>
+      <c r="D60" s="46"/>
+      <c r="E60" s="46"/>
     </row>
     <row r="61" ht="19.5" customHeight="1">
-      <c r="A61" s="46" t="s">
+      <c r="A61" s="45" t="s">
         <v>92</v>
       </c>
-      <c r="B61" s="48"/>
-      <c r="C61" s="48"/>
-      <c r="D61" s="48"/>
-      <c r="E61" s="48"/>
+      <c r="B61" s="47"/>
+      <c r="C61" s="47"/>
+      <c r="D61" s="47"/>
+      <c r="E61" s="47"/>
     </row>
     <row r="62" ht="19.5" customHeight="1">
-      <c r="A62" s="46" t="s">
+      <c r="A62" s="45" t="s">
         <v>195</v>
       </c>
-      <c r="B62" s="48"/>
-      <c r="C62" s="48"/>
-      <c r="D62" s="48"/>
-      <c r="E62" s="48"/>
+      <c r="B62" s="47"/>
+      <c r="C62" s="47"/>
+      <c r="D62" s="47"/>
+      <c r="E62" s="47"/>
     </row>
     <row r="63" ht="19.5" customHeight="1">
-      <c r="A63" s="46" t="s">
+      <c r="A63" s="45" t="s">
         <v>103</v>
       </c>
-      <c r="B63" s="48" t="s">
+      <c r="B63" s="47" t="s">
         <v>137</v>
       </c>
-      <c r="C63" s="48"/>
-      <c r="D63" s="48"/>
-      <c r="E63" s="48"/>
+      <c r="C63" s="47"/>
+      <c r="D63" s="47"/>
+      <c r="E63" s="47"/>
     </row>
     <row r="64" ht="19.5" customHeight="1">
-      <c r="A64" s="46" t="s">
+      <c r="A64" s="45" t="s">
         <v>106</v>
       </c>
-      <c r="B64" s="48"/>
-      <c r="C64" s="48"/>
-      <c r="D64" s="48"/>
-      <c r="E64" s="48"/>
+      <c r="B64" s="47"/>
+      <c r="C64" s="47"/>
+      <c r="D64" s="47"/>
+      <c r="E64" s="47"/>
     </row>
     <row r="65" ht="19.5" customHeight="1">
-      <c r="A65" s="46" t="s">
+      <c r="A65" s="45" t="s">
         <v>196</v>
       </c>
-      <c r="B65" s="48"/>
-      <c r="C65" s="48"/>
-      <c r="D65" s="48"/>
-      <c r="E65" s="48"/>
+      <c r="B65" s="47"/>
+      <c r="C65" s="47"/>
+      <c r="D65" s="47"/>
+      <c r="E65" s="47"/>
     </row>
     <row r="66" ht="6" customHeight="1"/>
     <row r="68" ht="15" customHeight="1">
-      <c r="A68" s="45" t="s">
+      <c r="A68" s="44" t="s">
         <v>201</v>
       </c>
-      <c r="B68" s="45"/>
-      <c r="C68" s="45"/>
-      <c r="D68" s="45"/>
-      <c r="E68" s="45"/>
+      <c r="B68" s="44"/>
+      <c r="C68" s="44"/>
+      <c r="D68" s="44"/>
+      <c r="E68" s="44"/>
     </row>
     <row r="69" ht="19.5" customHeight="1">
-      <c r="A69" s="46" t="s">
+      <c r="A69" s="45" t="s">
         <v>91</v>
       </c>
-      <c r="B69" s="47" t="s">
+      <c r="B69" s="46" t="s">
         <v>181</v>
       </c>
-      <c r="C69" s="47"/>
-      <c r="D69" s="47"/>
-      <c r="E69" s="47"/>
+      <c r="C69" s="46"/>
+      <c r="D69" s="46"/>
+      <c r="E69" s="46"/>
     </row>
     <row r="70" ht="19.5" customHeight="1">
-      <c r="A70" s="46" t="s">
+      <c r="A70" s="45" t="s">
         <v>92</v>
       </c>
-      <c r="B70" s="48"/>
-      <c r="C70" s="48"/>
-      <c r="D70" s="48"/>
-      <c r="E70" s="48"/>
+      <c r="B70" s="47"/>
+      <c r="C70" s="47"/>
+      <c r="D70" s="47"/>
+      <c r="E70" s="47"/>
     </row>
     <row r="71" ht="19.5" customHeight="1">
-      <c r="A71" s="46" t="s">
+      <c r="A71" s="45" t="s">
         <v>195</v>
       </c>
-      <c r="B71" s="48"/>
-      <c r="C71" s="48"/>
-      <c r="D71" s="48"/>
-      <c r="E71" s="48"/>
+      <c r="B71" s="47"/>
+      <c r="C71" s="47"/>
+      <c r="D71" s="47"/>
+      <c r="E71" s="47"/>
     </row>
     <row r="72" ht="19.5" customHeight="1">
-      <c r="A72" s="46" t="s">
+      <c r="A72" s="45" t="s">
         <v>103</v>
       </c>
-      <c r="B72" s="48" t="s">
+      <c r="B72" s="47" t="s">
         <v>137</v>
       </c>
-      <c r="C72" s="48"/>
-      <c r="D72" s="48"/>
-      <c r="E72" s="48"/>
+      <c r="C72" s="47"/>
+      <c r="D72" s="47"/>
+      <c r="E72" s="47"/>
     </row>
     <row r="73" ht="19.5" customHeight="1">
-      <c r="A73" s="46" t="s">
+      <c r="A73" s="45" t="s">
         <v>106</v>
       </c>
-      <c r="B73" s="48"/>
-      <c r="C73" s="48"/>
-      <c r="D73" s="48"/>
-      <c r="E73" s="48"/>
+      <c r="B73" s="47"/>
+      <c r="C73" s="47"/>
+      <c r="D73" s="47"/>
+      <c r="E73" s="47"/>
     </row>
     <row r="74" ht="19.5" customHeight="1">
-      <c r="A74" s="46" t="s">
+      <c r="A74" s="45" t="s">
         <v>196</v>
       </c>
-      <c r="B74" s="48"/>
-      <c r="C74" s="48"/>
-      <c r="D74" s="48"/>
-      <c r="E74" s="48"/>
+      <c r="B74" s="47"/>
+      <c r="C74" s="47"/>
+      <c r="D74" s="47"/>
+      <c r="E74" s="47"/>
     </row>
     <row r="75" ht="6" customHeight="1"/>
     <row r="77" ht="15" customHeight="1">
-      <c r="A77" s="45" t="s">
+      <c r="A77" s="44" t="s">
         <v>202</v>
       </c>
-      <c r="B77" s="45"/>
-      <c r="C77" s="45"/>
-      <c r="D77" s="45"/>
-      <c r="E77" s="45"/>
+      <c r="B77" s="44"/>
+      <c r="C77" s="44"/>
+      <c r="D77" s="44"/>
+      <c r="E77" s="44"/>
     </row>
     <row r="78" ht="19.5" customHeight="1">
-      <c r="A78" s="46" t="s">
+      <c r="A78" s="45" t="s">
         <v>91</v>
       </c>
-      <c r="B78" s="47" t="s">
+      <c r="B78" s="46" t="s">
         <v>183</v>
       </c>
-      <c r="C78" s="47"/>
-      <c r="D78" s="47"/>
-      <c r="E78" s="47"/>
+      <c r="C78" s="46"/>
+      <c r="D78" s="46"/>
+      <c r="E78" s="46"/>
     </row>
     <row r="79" ht="19.5" customHeight="1">
-      <c r="A79" s="46" t="s">
+      <c r="A79" s="45" t="s">
         <v>92</v>
       </c>
-      <c r="B79" s="48"/>
-      <c r="C79" s="48"/>
-      <c r="D79" s="48"/>
-      <c r="E79" s="48"/>
+      <c r="B79" s="47"/>
+      <c r="C79" s="47"/>
+      <c r="D79" s="47"/>
+      <c r="E79" s="47"/>
     </row>
     <row r="80" ht="19.5" customHeight="1">
-      <c r="A80" s="46" t="s">
+      <c r="A80" s="45" t="s">
         <v>195</v>
       </c>
-      <c r="B80" s="48"/>
-      <c r="C80" s="48"/>
-      <c r="D80" s="48"/>
-      <c r="E80" s="48"/>
+      <c r="B80" s="47"/>
+      <c r="C80" s="47"/>
+      <c r="D80" s="47"/>
+      <c r="E80" s="47"/>
     </row>
     <row r="81" ht="19.5" customHeight="1">
-      <c r="A81" s="46" t="s">
+      <c r="A81" s="45" t="s">
         <v>103</v>
       </c>
-      <c r="B81" s="48" t="s">
+      <c r="B81" s="47" t="s">
         <v>137</v>
       </c>
-      <c r="C81" s="48"/>
-      <c r="D81" s="48"/>
-      <c r="E81" s="48"/>
+      <c r="C81" s="47"/>
+      <c r="D81" s="47"/>
+      <c r="E81" s="47"/>
     </row>
     <row r="82" ht="19.5" customHeight="1">
-      <c r="A82" s="46" t="s">
+      <c r="A82" s="45" t="s">
         <v>106</v>
       </c>
-      <c r="B82" s="48"/>
-      <c r="C82" s="48"/>
-      <c r="D82" s="48"/>
-      <c r="E82" s="48"/>
+      <c r="B82" s="47"/>
+      <c r="C82" s="47"/>
+      <c r="D82" s="47"/>
+      <c r="E82" s="47"/>
     </row>
     <row r="83" ht="19.5" customHeight="1">
-      <c r="A83" s="46" t="s">
+      <c r="A83" s="45" t="s">
         <v>196</v>
       </c>
-      <c r="B83" s="48"/>
-      <c r="C83" s="48"/>
-      <c r="D83" s="48"/>
-      <c r="E83" s="48"/>
+      <c r="B83" s="47"/>
+      <c r="C83" s="47"/>
+      <c r="D83" s="47"/>
+      <c r="E83" s="47"/>
     </row>
     <row r="84" ht="6" customHeight="1"/>
     <row r="86" ht="15" customHeight="1">
-      <c r="A86" s="45" t="s">
+      <c r="A86" s="44" t="s">
         <v>203</v>
       </c>
-      <c r="B86" s="45"/>
-      <c r="C86" s="45"/>
-      <c r="D86" s="45"/>
-      <c r="E86" s="45"/>
+      <c r="B86" s="44"/>
+      <c r="C86" s="44"/>
+      <c r="D86" s="44"/>
+      <c r="E86" s="44"/>
     </row>
     <row r="87" ht="19.5" customHeight="1">
-      <c r="A87" s="46" t="s">
+      <c r="A87" s="45" t="s">
         <v>91</v>
       </c>
-      <c r="B87" s="47" t="s">
+      <c r="B87" s="46" t="s">
         <v>185</v>
       </c>
-      <c r="C87" s="47"/>
-      <c r="D87" s="47"/>
-      <c r="E87" s="47"/>
+      <c r="C87" s="46"/>
+      <c r="D87" s="46"/>
+      <c r="E87" s="46"/>
     </row>
     <row r="88" ht="19.5" customHeight="1">
-      <c r="A88" s="46" t="s">
+      <c r="A88" s="45" t="s">
         <v>92</v>
       </c>
-      <c r="B88" s="48"/>
-      <c r="C88" s="48"/>
-      <c r="D88" s="48"/>
-      <c r="E88" s="48"/>
+      <c r="B88" s="47"/>
+      <c r="C88" s="47"/>
+      <c r="D88" s="47"/>
+      <c r="E88" s="47"/>
     </row>
     <row r="89" ht="19.5" customHeight="1">
-      <c r="A89" s="46" t="s">
+      <c r="A89" s="45" t="s">
         <v>195</v>
       </c>
-      <c r="B89" s="48"/>
-      <c r="C89" s="48"/>
-      <c r="D89" s="48"/>
-      <c r="E89" s="48"/>
+      <c r="B89" s="47"/>
+      <c r="C89" s="47"/>
+      <c r="D89" s="47"/>
+      <c r="E89" s="47"/>
     </row>
     <row r="90" ht="19.5" customHeight="1">
-      <c r="A90" s="46" t="s">
+      <c r="A90" s="45" t="s">
         <v>103</v>
       </c>
-      <c r="B90" s="48" t="s">
+      <c r="B90" s="47" t="s">
         <v>137</v>
       </c>
-      <c r="C90" s="48"/>
-      <c r="D90" s="48"/>
-      <c r="E90" s="48"/>
+      <c r="C90" s="47"/>
+      <c r="D90" s="47"/>
+      <c r="E90" s="47"/>
     </row>
     <row r="91" ht="19.5" customHeight="1">
-      <c r="A91" s="46" t="s">
+      <c r="A91" s="45" t="s">
         <v>106</v>
       </c>
-      <c r="B91" s="48"/>
-      <c r="C91" s="48"/>
-      <c r="D91" s="48"/>
-      <c r="E91" s="48"/>
+      <c r="B91" s="47"/>
+      <c r="C91" s="47"/>
+      <c r="D91" s="47"/>
+      <c r="E91" s="47"/>
     </row>
     <row r="92" ht="19.5" customHeight="1">
-      <c r="A92" s="46" t="s">
+      <c r="A92" s="45" t="s">
         <v>196</v>
       </c>
-      <c r="B92" s="48"/>
-      <c r="C92" s="48"/>
-      <c r="D92" s="48"/>
-      <c r="E92" s="48"/>
+      <c r="B92" s="47"/>
+      <c r="C92" s="47"/>
+      <c r="D92" s="47"/>
+      <c r="E92" s="47"/>
     </row>
     <row r="93" ht="6" customHeight="1"/>
     <row r="95" ht="15" customHeight="1">
-      <c r="A95" s="45" t="s">
+      <c r="A95" s="44" t="s">
         <v>204</v>
       </c>
-      <c r="B95" s="45"/>
-      <c r="C95" s="45"/>
-      <c r="D95" s="45"/>
-      <c r="E95" s="45"/>
+      <c r="B95" s="44"/>
+      <c r="C95" s="44"/>
+      <c r="D95" s="44"/>
+      <c r="E95" s="44"/>
     </row>
     <row r="96" ht="19.5" customHeight="1">
-      <c r="A96" s="46" t="s">
+      <c r="A96" s="45" t="s">
         <v>91</v>
       </c>
-      <c r="B96" s="47" t="s">
+      <c r="B96" s="46" t="s">
         <v>187</v>
       </c>
-      <c r="C96" s="47"/>
-      <c r="D96" s="47"/>
-      <c r="E96" s="47"/>
+      <c r="C96" s="46"/>
+      <c r="D96" s="46"/>
+      <c r="E96" s="46"/>
     </row>
     <row r="97" ht="19.5" customHeight="1">
-      <c r="A97" s="46" t="s">
+      <c r="A97" s="45" t="s">
         <v>92</v>
       </c>
-      <c r="B97" s="48"/>
-      <c r="C97" s="48"/>
-      <c r="D97" s="48"/>
-      <c r="E97" s="48"/>
+      <c r="B97" s="47"/>
+      <c r="C97" s="47"/>
+      <c r="D97" s="47"/>
+      <c r="E97" s="47"/>
     </row>
     <row r="98" ht="19.5" customHeight="1">
-      <c r="A98" s="46" t="s">
+      <c r="A98" s="45" t="s">
         <v>195</v>
       </c>
-      <c r="B98" s="48"/>
-      <c r="C98" s="48"/>
-      <c r="D98" s="48"/>
-      <c r="E98" s="48"/>
+      <c r="B98" s="47"/>
+      <c r="C98" s="47"/>
+      <c r="D98" s="47"/>
+      <c r="E98" s="47"/>
     </row>
     <row r="99" ht="19.5" customHeight="1">
-      <c r="A99" s="46" t="s">
+      <c r="A99" s="45" t="s">
         <v>103</v>
       </c>
-      <c r="B99" s="48" t="s">
+      <c r="B99" s="47" t="s">
         <v>137</v>
       </c>
-      <c r="C99" s="48"/>
-      <c r="D99" s="48"/>
-      <c r="E99" s="48"/>
+      <c r="C99" s="47"/>
+      <c r="D99" s="47"/>
+      <c r="E99" s="47"/>
     </row>
     <row r="100" ht="19.5" customHeight="1">
-      <c r="A100" s="46" t="s">
+      <c r="A100" s="45" t="s">
         <v>106</v>
       </c>
-      <c r="B100" s="48"/>
-      <c r="C100" s="48"/>
-      <c r="D100" s="48"/>
-      <c r="E100" s="48"/>
+      <c r="B100" s="47"/>
+      <c r="C100" s="47"/>
+      <c r="D100" s="47"/>
+      <c r="E100" s="47"/>
     </row>
     <row r="101" ht="19.5" customHeight="1">
-      <c r="A101" s="46" t="s">
+      <c r="A101" s="45" t="s">
         <v>196</v>
       </c>
-      <c r="B101" s="48"/>
-      <c r="C101" s="48"/>
-      <c r="D101" s="48"/>
-      <c r="E101" s="48"/>
+      <c r="B101" s="47"/>
+      <c r="C101" s="47"/>
+      <c r="D101" s="47"/>
+      <c r="E101" s="47"/>
     </row>
     <row r="102" ht="6" customHeight="1"/>
     <row r="104" ht="15" customHeight="1">
-      <c r="A104" s="45" t="s">
+      <c r="A104" s="44" t="s">
         <v>205</v>
       </c>
-      <c r="B104" s="45"/>
-      <c r="C104" s="45"/>
-      <c r="D104" s="45"/>
-      <c r="E104" s="45"/>
+      <c r="B104" s="44"/>
+      <c r="C104" s="44"/>
+      <c r="D104" s="44"/>
+      <c r="E104" s="44"/>
     </row>
     <row r="105" ht="19.5" customHeight="1">
-      <c r="A105" s="46" t="s">
+      <c r="A105" s="45" t="s">
         <v>91</v>
       </c>
-      <c r="B105" s="47" t="s">
+      <c r="B105" s="46" t="s">
         <v>189</v>
       </c>
-      <c r="C105" s="47"/>
-      <c r="D105" s="47"/>
-      <c r="E105" s="47"/>
+      <c r="C105" s="46"/>
+      <c r="D105" s="46"/>
+      <c r="E105" s="46"/>
     </row>
     <row r="106" ht="19.5" customHeight="1">
-      <c r="A106" s="46" t="s">
+      <c r="A106" s="45" t="s">
         <v>92</v>
       </c>
-      <c r="B106" s="48"/>
-      <c r="C106" s="48"/>
-      <c r="D106" s="48"/>
-      <c r="E106" s="48"/>
+      <c r="B106" s="47"/>
+      <c r="C106" s="47"/>
+      <c r="D106" s="47"/>
+      <c r="E106" s="47"/>
     </row>
     <row r="107" ht="19.5" customHeight="1">
-      <c r="A107" s="46" t="s">
+      <c r="A107" s="45" t="s">
         <v>195</v>
       </c>
-      <c r="B107" s="48"/>
-      <c r="C107" s="48"/>
-      <c r="D107" s="48"/>
-      <c r="E107" s="48"/>
+      <c r="B107" s="47"/>
+      <c r="C107" s="47"/>
+      <c r="D107" s="47"/>
+      <c r="E107" s="47"/>
     </row>
     <row r="108" ht="19.5" customHeight="1">
-      <c r="A108" s="46" t="s">
+      <c r="A108" s="45" t="s">
         <v>103</v>
       </c>
-      <c r="B108" s="48" t="s">
+      <c r="B108" s="47" t="s">
         <v>137</v>
       </c>
-      <c r="C108" s="48"/>
-      <c r="D108" s="48"/>
-      <c r="E108" s="48"/>
+      <c r="C108" s="47"/>
+      <c r="D108" s="47"/>
+      <c r="E108" s="47"/>
     </row>
     <row r="109" ht="19.5" customHeight="1">
-      <c r="A109" s="46" t="s">
+      <c r="A109" s="45" t="s">
         <v>106</v>
       </c>
-      <c r="B109" s="48"/>
-      <c r="C109" s="48"/>
-      <c r="D109" s="48"/>
-      <c r="E109" s="48"/>
+      <c r="B109" s="47"/>
+      <c r="C109" s="47"/>
+      <c r="D109" s="47"/>
+      <c r="E109" s="47"/>
     </row>
     <row r="110" ht="19.5" customHeight="1">
-      <c r="A110" s="46" t="s">
+      <c r="A110" s="45" t="s">
         <v>196</v>
       </c>
-      <c r="B110" s="48"/>
-      <c r="C110" s="48"/>
-      <c r="D110" s="48"/>
-      <c r="E110" s="48"/>
+      <c r="B110" s="47"/>
+      <c r="C110" s="47"/>
+      <c r="D110" s="47"/>
+      <c r="E110" s="47"/>
     </row>
     <row r="111" ht="6" customHeight="1"/>
     <row r="113" ht="15" customHeight="1">
-      <c r="A113" s="45" t="s">
+      <c r="A113" s="44" t="s">
         <v>206</v>
       </c>
-      <c r="B113" s="45"/>
-      <c r="C113" s="45"/>
-      <c r="D113" s="45"/>
-      <c r="E113" s="45"/>
+      <c r="B113" s="44"/>
+      <c r="C113" s="44"/>
+      <c r="D113" s="44"/>
+      <c r="E113" s="44"/>
     </row>
     <row r="114" ht="19.5" customHeight="1">
-      <c r="A114" s="46" t="s">
+      <c r="A114" s="45" t="s">
         <v>91</v>
       </c>
-      <c r="B114" s="47" t="s">
+      <c r="B114" s="46" t="s">
         <v>191</v>
       </c>
-      <c r="C114" s="47"/>
-      <c r="D114" s="47"/>
-      <c r="E114" s="47"/>
+      <c r="C114" s="46"/>
+      <c r="D114" s="46"/>
+      <c r="E114" s="46"/>
     </row>
     <row r="115" ht="19.5" customHeight="1">
-      <c r="A115" s="46" t="s">
+      <c r="A115" s="45" t="s">
         <v>92</v>
       </c>
-      <c r="B115" s="48"/>
-      <c r="C115" s="48"/>
-      <c r="D115" s="48"/>
-      <c r="E115" s="48"/>
+      <c r="B115" s="47"/>
+      <c r="C115" s="47"/>
+      <c r="D115" s="47"/>
+      <c r="E115" s="47"/>
     </row>
     <row r="116" ht="19.5" customHeight="1">
-      <c r="A116" s="46" t="s">
+      <c r="A116" s="45" t="s">
         <v>195</v>
       </c>
-      <c r="B116" s="48"/>
-      <c r="C116" s="48"/>
-      <c r="D116" s="48"/>
-      <c r="E116" s="48"/>
+      <c r="B116" s="47"/>
+      <c r="C116" s="47"/>
+      <c r="D116" s="47"/>
+      <c r="E116" s="47"/>
     </row>
     <row r="117" ht="19.5" customHeight="1">
-      <c r="A117" s="46" t="s">
+      <c r="A117" s="45" t="s">
         <v>103</v>
       </c>
-      <c r="B117" s="48" t="s">
+      <c r="B117" s="47" t="s">
         <v>137</v>
       </c>
-      <c r="C117" s="48"/>
-      <c r="D117" s="48"/>
-      <c r="E117" s="48"/>
+      <c r="C117" s="47"/>
+      <c r="D117" s="47"/>
+      <c r="E117" s="47"/>
     </row>
     <row r="118" ht="19.5" customHeight="1">
-      <c r="A118" s="46" t="s">
+      <c r="A118" s="45" t="s">
         <v>106</v>
       </c>
-      <c r="B118" s="48"/>
-      <c r="C118" s="48"/>
-      <c r="D118" s="48"/>
-      <c r="E118" s="48"/>
+      <c r="B118" s="47"/>
+      <c r="C118" s="47"/>
+      <c r="D118" s="47"/>
+      <c r="E118" s="47"/>
     </row>
     <row r="119" ht="19.5" customHeight="1">
-      <c r="A119" s="46" t="s">
+      <c r="A119" s="45" t="s">
         <v>196</v>
       </c>
-      <c r="B119" s="48"/>
-      <c r="C119" s="48"/>
-      <c r="D119" s="48"/>
-      <c r="E119" s="48"/>
+      <c r="B119" s="47"/>
+      <c r="C119" s="47"/>
+      <c r="D119" s="47"/>
+      <c r="E119" s="47"/>
     </row>
     <row r="120" ht="6" customHeight="1"/>
     <row r="122" ht="15" customHeight="1">
-      <c r="A122" s="45" t="s">
+      <c r="A122" s="44" t="s">
         <v>207</v>
       </c>
-      <c r="B122" s="45"/>
-      <c r="C122" s="45"/>
-      <c r="D122" s="45"/>
-      <c r="E122" s="45"/>
+      <c r="B122" s="44"/>
+      <c r="C122" s="44"/>
+      <c r="D122" s="44"/>
+      <c r="E122" s="44"/>
     </row>
     <row r="123" ht="19.5" customHeight="1">
-      <c r="A123" s="46" t="s">
+      <c r="A123" s="45" t="s">
         <v>91</v>
       </c>
-      <c r="B123" s="47" t="s">
+      <c r="B123" s="46" t="s">
         <v>193</v>
       </c>
-      <c r="C123" s="47"/>
-      <c r="D123" s="47"/>
-      <c r="E123" s="47"/>
+      <c r="C123" s="46"/>
+      <c r="D123" s="46"/>
+      <c r="E123" s="46"/>
     </row>
     <row r="124" ht="19.5" customHeight="1">
-      <c r="A124" s="46" t="s">
+      <c r="A124" s="45" t="s">
         <v>92</v>
       </c>
-      <c r="B124" s="48"/>
-      <c r="C124" s="48"/>
-      <c r="D124" s="48"/>
-      <c r="E124" s="48"/>
+      <c r="B124" s="47"/>
+      <c r="C124" s="47"/>
+      <c r="D124" s="47"/>
+      <c r="E124" s="47"/>
     </row>
     <row r="125" ht="19.5" customHeight="1">
-      <c r="A125" s="46" t="s">
+      <c r="A125" s="45" t="s">
         <v>195</v>
       </c>
-      <c r="B125" s="48"/>
-      <c r="C125" s="48"/>
-      <c r="D125" s="48"/>
-      <c r="E125" s="48"/>
+      <c r="B125" s="47"/>
+      <c r="C125" s="47"/>
+      <c r="D125" s="47"/>
+      <c r="E125" s="47"/>
     </row>
     <row r="126" ht="19.5" customHeight="1">
-      <c r="A126" s="46" t="s">
+      <c r="A126" s="45" t="s">
         <v>103</v>
       </c>
-      <c r="B126" s="48" t="s">
+      <c r="B126" s="47" t="s">
         <v>137</v>
       </c>
-      <c r="C126" s="48"/>
-      <c r="D126" s="48"/>
-      <c r="E126" s="48"/>
+      <c r="C126" s="47"/>
+      <c r="D126" s="47"/>
+      <c r="E126" s="47"/>
     </row>
     <row r="127" ht="19.5" customHeight="1">
-      <c r="A127" s="46" t="s">
+      <c r="A127" s="45" t="s">
         <v>106</v>
       </c>
-      <c r="B127" s="48"/>
-      <c r="C127" s="48"/>
-      <c r="D127" s="48"/>
-      <c r="E127" s="48"/>
+      <c r="B127" s="47"/>
+      <c r="C127" s="47"/>
+      <c r="D127" s="47"/>
+      <c r="E127" s="47"/>
     </row>
     <row r="128" ht="19.5" customHeight="1">
-      <c r="A128" s="46" t="s">
+      <c r="A128" s="45" t="s">
         <v>196</v>
       </c>
-      <c r="B128" s="48"/>
-      <c r="C128" s="48"/>
-      <c r="D128" s="48"/>
-      <c r="E128" s="48"/>
+      <c r="B128" s="47"/>
+      <c r="C128" s="47"/>
+      <c r="D128" s="47"/>
+      <c r="E128" s="47"/>
     </row>
     <row r="129" ht="6" customHeight="1"/>
   </sheetData>
@@ -5049,7 +5048,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="6"/>
     <col customWidth="1" min="2" max="2" width="13"/>
@@ -5090,22 +5089,22 @@
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="41">
+      <c r="A4" s="40">
         <v>1</v>
       </c>
-      <c r="B4" s="49">
+      <c r="B4" s="48">
         <v>46168</v>
       </c>
-      <c r="C4" s="42" t="s">
+      <c r="C4" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="50" t="s">
+      <c r="D4" s="49" t="s">
         <v>215</v>
       </c>
-      <c r="E4" s="42" t="s">
+      <c r="E4" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="42" t="str">
+      <c r="F4" s="41" t="str">
         <f t="shared" ref="F4:F9" si="4">IF(ISBLANK(B4),"offen","fertig")</f>
         <v>fertig</v>
       </c>
@@ -5114,7 +5113,7 @@
       <c r="A5" s="8">
         <v>2</v>
       </c>
-      <c r="B5" s="49">
+      <c r="B5" s="48">
         <v>46170</v>
       </c>
       <c r="C5" s="10" t="s">
@@ -5126,28 +5125,28 @@
       <c r="E5" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="42" t="str">
+      <c r="F5" s="41" t="str">
         <f t="shared" si="4"/>
         <v>fertig</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
-      <c r="A6" s="41">
+      <c r="A6" s="40">
         <v>3</v>
       </c>
       <c r="B6" s="35">
         <v>46175</v>
       </c>
-      <c r="C6" s="42" t="s">
+      <c r="C6" s="41" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="50" t="s">
+      <c r="D6" s="49" t="s">
         <v>217</v>
       </c>
-      <c r="E6" s="42" t="s">
+      <c r="E6" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="F6" s="42" t="str">
+      <c r="F6" s="41" t="str">
         <f t="shared" si="4"/>
         <v>fertig</v>
       </c>
@@ -5168,26 +5167,26 @@
       <c r="E7" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="F7" s="42" t="str">
+      <c r="F7" s="41" t="str">
         <f t="shared" si="4"/>
         <v>fertig</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="41">
+      <c r="A8" s="40">
         <v>5</v>
       </c>
       <c r="B8" s="35"/>
-      <c r="C8" s="42" t="s">
+      <c r="C8" s="41" t="s">
         <v>220</v>
       </c>
-      <c r="D8" s="50" t="s">
+      <c r="D8" s="49" t="s">
         <v>221</v>
       </c>
-      <c r="E8" s="42" t="s">
+      <c r="E8" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="42" t="str">
+      <c r="F8" s="41" t="str">
         <f t="shared" si="4"/>
         <v>offen</v>
       </c>
@@ -5206,7 +5205,7 @@
       <c r="E9" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="F9" s="42" t="str">
+      <c r="F9" s="41" t="str">
         <f t="shared" si="4"/>
         <v>offen</v>
       </c>
@@ -5230,127 +5229,127 @@
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="50" t="s">
         <v>224</v>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="52"/>
+      <c r="A5" s="51"/>
     </row>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="53" t="s">
+      <c r="A6" s="52" t="s">
         <v>225</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="52" t="s">
+      <c r="A7" s="51" t="s">
         <v>226</v>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="A8" s="52" t="s">
+      <c r="A8" s="51" t="s">
         <v>227</v>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
-      <c r="A9" s="52" t="s">
+      <c r="A9" s="51" t="s">
         <v>228</v>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
-      <c r="A10" s="52" t="s">
+      <c r="A10" s="51" t="s">
         <v>229</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="52" t="s">
+      <c r="A11" s="51" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
-      <c r="A12" s="52"/>
+      <c r="A12" s="51"/>
     </row>
     <row r="13" ht="15.75" customHeight="1">
-      <c r="A13" s="53" t="s">
+      <c r="A13" s="52" t="s">
         <v>231</v>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
-      <c r="A14" s="52" t="s">
+      <c r="A14" s="51" t="s">
         <v>232</v>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1">
-      <c r="A15" s="52" t="s">
+      <c r="A15" s="51" t="s">
         <v>233</v>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
-      <c r="A16" s="52" t="s">
+      <c r="A16" s="51" t="s">
         <v>234</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
-      <c r="A17" s="52" t="s">
+      <c r="A17" s="51" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
-      <c r="A18" s="52"/>
+      <c r="A18" s="51"/>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="53" t="s">
+      <c r="A19" s="52" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="52" t="s">
+      <c r="A20" s="51" t="s">
         <v>237</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="52" t="s">
+      <c r="A21" s="51" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="52"/>
+      <c r="A22" s="51"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="53" t="s">
+      <c r="A23" s="52" t="s">
         <v>239</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="52" t="s">
+      <c r="A24" s="51" t="s">
         <v>240</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="52" t="s">
+      <c r="A25" s="51" t="s">
         <v>241</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="52" t="s">
+      <c r="A26" s="51" t="s">
         <v>242</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="52"/>
+      <c r="A27" s="51"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="53" t="s">
+      <c r="A28" s="52" t="s">
         <v>243</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="52" t="s">
+      <c r="A29" s="51" t="s">
         <v>244</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="52" t="s">
+      <c r="A30" s="51" t="s">
         <v>245</v>
       </c>
     </row>

</xml_diff>

<commit_message>
v.0.47 Update Docker for production
</commit_message>
<xml_diff>
--- a/docs/PSP_OnlineShop.xlsx
+++ b/docs/PSP_OnlineShop.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="2"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="PSP" sheetId="1" state="visible" r:id="rId1"/>
@@ -1054,6 +1054,9 @@
     <xf fontId="3" fillId="3" borderId="1" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf fontId="0" fillId="8" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf fontId="3" fillId="10" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1062,9 +1065,6 @@
     </xf>
     <xf fontId="0" fillId="8" borderId="1" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="8" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="4" fillId="6" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2884,7 +2884,9 @@
       <c r="A100" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="B100" s="31"/>
+      <c r="B100" s="29">
+        <v>46192</v>
+      </c>
     </row>
     <row r="101" ht="19.5" customHeight="1">
       <c r="A101" s="27" t="s">
@@ -2957,7 +2959,7 @@
         <v>102</v>
       </c>
       <c r="B110" s="29">
-        <v>46182</v>
+        <v>46192</v>
       </c>
     </row>
     <row r="111" ht="19.5" customHeight="1">
@@ -2972,7 +2974,9 @@
       <c r="A112" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="B112" s="31"/>
+      <c r="B112" s="29">
+        <v>46193</v>
+      </c>
     </row>
     <row r="113" ht="19.5" customHeight="1">
       <c r="A113" s="27" t="s">
@@ -3646,14 +3650,16 @@
       <c r="F25" s="34">
         <v>46206</v>
       </c>
-      <c r="G25" s="35"/>
-      <c r="H25" s="36" t="str">
+      <c r="G25" s="35">
+        <v>46191</v>
+      </c>
+      <c r="H25" s="36">
         <f t="shared" si="0"/>
-        <v/>
+        <v>-15</v>
       </c>
       <c r="I25" s="37" t="str">
         <f t="shared" si="1"/>
-        <v>offen</v>
+        <v>fertig</v>
       </c>
       <c r="J25" s="19"/>
     </row>
@@ -3676,14 +3682,16 @@
       <c r="F26" s="39">
         <v>46210</v>
       </c>
-      <c r="G26" s="35"/>
-      <c r="H26" s="36" t="str">
+      <c r="G26" s="35">
+        <v>46192</v>
+      </c>
+      <c r="H26" s="36">
         <f t="shared" si="0"/>
-        <v/>
+        <v>-18</v>
       </c>
       <c r="I26" s="37" t="str">
         <f t="shared" si="1"/>
-        <v>offen</v>
+        <v>fertig</v>
       </c>
       <c r="J26" s="9"/>
     </row>
@@ -3706,14 +3714,16 @@
       <c r="F27" s="39">
         <v>46212</v>
       </c>
-      <c r="G27" s="35"/>
-      <c r="H27" s="36" t="str">
+      <c r="G27" s="35">
+        <v>46193</v>
+      </c>
+      <c r="H27" s="36">
         <f t="shared" si="0"/>
-        <v/>
+        <v>-19</v>
       </c>
       <c r="I27" s="37" t="str">
         <f t="shared" si="1"/>
-        <v>offen</v>
+        <v>fertig</v>
       </c>
       <c r="J27" s="9"/>
     </row>
@@ -3736,14 +3746,16 @@
       <c r="F28" s="38">
         <v>46212</v>
       </c>
-      <c r="G28" s="35"/>
-      <c r="H28" s="36" t="str">
+      <c r="G28" s="40">
+        <v>46193</v>
+      </c>
+      <c r="H28" s="36">
         <f t="shared" si="0"/>
-        <v/>
+        <v>-19</v>
       </c>
       <c r="I28" s="37" t="str">
         <f t="shared" si="1"/>
-        <v>offen</v>
+        <v>fertig</v>
       </c>
       <c r="J28" s="14"/>
     </row>
@@ -3961,10 +3973,10 @@
       </c>
     </row>
     <row r="8" ht="19.5" customHeight="1">
-      <c r="A8" s="40" t="s">
+      <c r="A8" s="41" t="s">
         <v>170</v>
       </c>
-      <c r="B8" s="41" t="s">
+      <c r="B8" s="42" t="s">
         <v>171</v>
       </c>
       <c r="C8" s="35">
@@ -3974,7 +3986,7 @@
         <f t="shared" ref="D8:D9" si="2">IF(ISBLANK(C8),"offen","fertig")</f>
         <v>fertig</v>
       </c>
-      <c r="E8" s="42"/>
+      <c r="E8" s="43"/>
     </row>
     <row r="9" ht="19.5" customHeight="1">
       <c r="A9" s="8" t="s">
@@ -3990,23 +4002,23 @@
         <f t="shared" si="2"/>
         <v>fertig</v>
       </c>
-      <c r="E9" s="42"/>
+      <c r="E9" s="43"/>
     </row>
     <row r="10" ht="19.5" customHeight="1">
-      <c r="A10" s="40" t="s">
+      <c r="A10" s="41" t="s">
         <v>174</v>
       </c>
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="42" t="s">
         <v>175</v>
       </c>
-      <c r="C10" s="43">
+      <c r="C10" s="40">
         <v>46177</v>
       </c>
       <c r="D10" s="37" t="str">
         <f t="shared" ref="D10:D19" si="3">IF(ISBLANK(C10),"offen","fertig")</f>
         <v>fertig</v>
       </c>
-      <c r="E10" s="42"/>
+      <c r="E10" s="43"/>
     </row>
     <row r="11" ht="19.5" customHeight="1">
       <c r="A11" s="8" t="s">
@@ -4015,26 +4027,30 @@
       <c r="B11" s="10" t="s">
         <v>177</v>
       </c>
-      <c r="C11" s="35"/>
+      <c r="C11" s="35">
+        <v>46179</v>
+      </c>
       <c r="D11" s="37" t="str">
         <f t="shared" si="3"/>
-        <v>offen</v>
-      </c>
-      <c r="E11" s="42"/>
+        <v>fertig</v>
+      </c>
+      <c r="E11" s="43"/>
     </row>
     <row r="12" ht="19.5" customHeight="1">
-      <c r="A12" s="40" t="s">
+      <c r="A12" s="41" t="s">
         <v>178</v>
       </c>
-      <c r="B12" s="41" t="s">
+      <c r="B12" s="42" t="s">
         <v>179</v>
       </c>
-      <c r="C12" s="35"/>
+      <c r="C12" s="35">
+        <v>46179</v>
+      </c>
       <c r="D12" s="37" t="str">
         <f t="shared" si="3"/>
-        <v>offen</v>
-      </c>
-      <c r="E12" s="42"/>
+        <v>fertig</v>
+      </c>
+      <c r="E12" s="43"/>
     </row>
     <row r="13" ht="19.5" customHeight="1">
       <c r="A13" s="8" t="s">
@@ -4043,26 +4059,30 @@
       <c r="B13" s="10" t="s">
         <v>181</v>
       </c>
-      <c r="C13" s="35"/>
+      <c r="C13" s="35">
+        <v>46184</v>
+      </c>
       <c r="D13" s="37" t="str">
         <f t="shared" si="3"/>
-        <v>offen</v>
-      </c>
-      <c r="E13" s="42"/>
+        <v>fertig</v>
+      </c>
+      <c r="E13" s="43"/>
     </row>
     <row r="14" ht="19.5" customHeight="1">
-      <c r="A14" s="40" t="s">
+      <c r="A14" s="41" t="s">
         <v>182</v>
       </c>
-      <c r="B14" s="41" t="s">
+      <c r="B14" s="42" t="s">
         <v>183</v>
       </c>
-      <c r="C14" s="35"/>
+      <c r="C14" s="35">
+        <v>46186</v>
+      </c>
       <c r="D14" s="37" t="str">
         <f t="shared" si="3"/>
-        <v>offen</v>
-      </c>
-      <c r="E14" s="42"/>
+        <v>fertig</v>
+      </c>
+      <c r="E14" s="43"/>
     </row>
     <row r="15" ht="19.5" customHeight="1">
       <c r="A15" s="8" t="s">
@@ -4071,26 +4091,30 @@
       <c r="B15" s="10" t="s">
         <v>185</v>
       </c>
-      <c r="C15" s="35"/>
+      <c r="C15" s="35">
+        <v>46187</v>
+      </c>
       <c r="D15" s="37" t="str">
         <f t="shared" si="3"/>
-        <v>offen</v>
-      </c>
-      <c r="E15" s="42"/>
+        <v>fertig</v>
+      </c>
+      <c r="E15" s="43"/>
     </row>
     <row r="16" ht="19.5" customHeight="1">
-      <c r="A16" s="40" t="s">
+      <c r="A16" s="41" t="s">
         <v>186</v>
       </c>
-      <c r="B16" s="41" t="s">
+      <c r="B16" s="42" t="s">
         <v>187</v>
       </c>
-      <c r="C16" s="35"/>
+      <c r="C16" s="35">
+        <v>46187</v>
+      </c>
       <c r="D16" s="37" t="str">
         <f t="shared" si="3"/>
-        <v>offen</v>
-      </c>
-      <c r="E16" s="42"/>
+        <v>fertig</v>
+      </c>
+      <c r="E16" s="43"/>
     </row>
     <row r="17" ht="19.5" customHeight="1">
       <c r="A17" s="8" t="s">
@@ -4099,26 +4123,30 @@
       <c r="B17" s="10" t="s">
         <v>189</v>
       </c>
-      <c r="C17" s="35"/>
+      <c r="C17" s="35">
+        <v>46189</v>
+      </c>
       <c r="D17" s="37" t="str">
         <f t="shared" si="3"/>
-        <v>offen</v>
-      </c>
-      <c r="E17" s="42"/>
+        <v>fertig</v>
+      </c>
+      <c r="E17" s="43"/>
     </row>
     <row r="18" ht="19.5" customHeight="1">
-      <c r="A18" s="40" t="s">
+      <c r="A18" s="41" t="s">
         <v>190</v>
       </c>
-      <c r="B18" s="41" t="s">
+      <c r="B18" s="42" t="s">
         <v>191</v>
       </c>
-      <c r="C18" s="35"/>
+      <c r="C18" s="35">
+        <v>46181</v>
+      </c>
       <c r="D18" s="37" t="str">
         <f t="shared" si="3"/>
-        <v>offen</v>
-      </c>
-      <c r="E18" s="42"/>
+        <v>fertig</v>
+      </c>
+      <c r="E18" s="43"/>
     </row>
     <row r="19" ht="19.5" customHeight="1">
       <c r="A19" s="8" t="s">
@@ -4127,12 +4155,14 @@
       <c r="B19" s="10" t="s">
         <v>193</v>
       </c>
-      <c r="C19" s="35"/>
+      <c r="C19" s="35">
+        <v>46178</v>
+      </c>
       <c r="D19" s="37" t="str">
         <f t="shared" si="3"/>
-        <v>offen</v>
-      </c>
-      <c r="E19" s="42"/>
+        <v>fertig</v>
+      </c>
+      <c r="E19" s="43"/>
     </row>
     <row r="22" ht="6" customHeight="1"/>
     <row r="23" ht="15" customHeight="1">
@@ -5089,22 +5119,22 @@
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="40">
+      <c r="A4" s="41">
         <v>1</v>
       </c>
       <c r="B4" s="48">
         <v>46168</v>
       </c>
-      <c r="C4" s="41" t="s">
+      <c r="C4" s="42" t="s">
         <v>17</v>
       </c>
       <c r="D4" s="49" t="s">
         <v>215</v>
       </c>
-      <c r="E4" s="41" t="s">
+      <c r="E4" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="41" t="str">
+      <c r="F4" s="42" t="str">
         <f t="shared" ref="F4:F9" si="4">IF(ISBLANK(B4),"offen","fertig")</f>
         <v>fertig</v>
       </c>
@@ -5125,28 +5155,28 @@
       <c r="E5" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="41" t="str">
+      <c r="F5" s="42" t="str">
         <f t="shared" si="4"/>
         <v>fertig</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
-      <c r="A6" s="40">
+      <c r="A6" s="41">
         <v>3</v>
       </c>
       <c r="B6" s="35">
         <v>46175</v>
       </c>
-      <c r="C6" s="41" t="s">
+      <c r="C6" s="42" t="s">
         <v>33</v>
       </c>
       <c r="D6" s="49" t="s">
         <v>217</v>
       </c>
-      <c r="E6" s="41" t="s">
+      <c r="E6" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="F6" s="41" t="str">
+      <c r="F6" s="42" t="str">
         <f t="shared" si="4"/>
         <v>fertig</v>
       </c>
@@ -5167,35 +5197,39 @@
       <c r="E7" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="F7" s="41" t="str">
+      <c r="F7" s="42" t="str">
         <f t="shared" si="4"/>
         <v>fertig</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="40">
+      <c r="A8" s="41">
         <v>5</v>
       </c>
-      <c r="B8" s="35"/>
-      <c r="C8" s="41" t="s">
+      <c r="B8" s="35">
+        <v>46193</v>
+      </c>
+      <c r="C8" s="42" t="s">
         <v>220</v>
       </c>
       <c r="D8" s="49" t="s">
         <v>221</v>
       </c>
-      <c r="E8" s="41" t="s">
+      <c r="E8" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="41" t="str">
+      <c r="F8" s="42" t="str">
         <f t="shared" si="4"/>
-        <v>offen</v>
+        <v>fertig</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="8">
         <v>6</v>
       </c>
-      <c r="B9" s="35"/>
+      <c r="B9" s="35">
+        <v>46194</v>
+      </c>
       <c r="C9" s="10" t="s">
         <v>222</v>
       </c>
@@ -5205,9 +5239,9 @@
       <c r="E9" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="F9" s="41" t="str">
+      <c r="F9" s="42" t="str">
         <f t="shared" si="4"/>
-        <v>offen</v>
+        <v>fertig</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v.1.0 Delete UML_OnlineShop.html Add UML_OnlineShop.md Add Projektabschlussbericht_OnlineShop.docx
</commit_message>
<xml_diff>
--- a/docs/PSP_OnlineShop.xlsx
+++ b/docs/PSP_OnlineShop.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="PSP" sheetId="1" state="visible" r:id="rId1"/>
@@ -3778,14 +3778,16 @@
       <c r="F29" s="34">
         <v>46213</v>
       </c>
-      <c r="G29" s="35"/>
-      <c r="H29" s="36" t="str">
+      <c r="G29" s="35">
+        <v>46194</v>
+      </c>
+      <c r="H29" s="36">
         <f t="shared" si="0"/>
-        <v/>
+        <v>-19</v>
       </c>
       <c r="I29" s="37" t="str">
         <f t="shared" si="1"/>
-        <v>offen</v>
+        <v>fertig</v>
       </c>
       <c r="J29" s="19"/>
     </row>
@@ -3808,14 +3810,16 @@
       <c r="F30" s="34">
         <v>46216</v>
       </c>
-      <c r="G30" s="35"/>
-      <c r="H30" s="36" t="str">
+      <c r="G30" s="35">
+        <v>46195</v>
+      </c>
+      <c r="H30" s="36">
         <f t="shared" si="0"/>
-        <v/>
+        <v>-21</v>
       </c>
       <c r="I30" s="37" t="str">
         <f t="shared" si="1"/>
-        <v>offen</v>
+        <v>fertig</v>
       </c>
       <c r="J30" s="19"/>
     </row>
@@ -3838,14 +3842,16 @@
       <c r="F31" s="38">
         <v>46217</v>
       </c>
-      <c r="G31" s="35"/>
-      <c r="H31" s="36" t="str">
+      <c r="G31" s="35">
+        <v>46195</v>
+      </c>
+      <c r="H31" s="36">
         <f t="shared" si="0"/>
-        <v/>
+        <v>-22</v>
       </c>
       <c r="I31" s="37" t="str">
         <f t="shared" si="1"/>
-        <v>offen</v>
+        <v>fertig</v>
       </c>
       <c r="J31" s="14" t="s">
         <v>165</v>
@@ -3870,14 +3876,16 @@
       <c r="F32" s="38">
         <v>46220</v>
       </c>
-      <c r="G32" s="35"/>
-      <c r="H32" s="36" t="str">
+      <c r="G32" s="35">
+        <v>46195</v>
+      </c>
+      <c r="H32" s="36">
         <f t="shared" si="0"/>
-        <v/>
+        <v>-25</v>
       </c>
       <c r="I32" s="37" t="str">
         <f t="shared" si="1"/>
-        <v>offen</v>
+        <v>fertig</v>
       </c>
       <c r="J32" s="14" t="s">
         <v>87</v>

</xml_diff>